<commit_message>
Safely purge 0001-0008 data without destroying metadata
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -851,11 +851,6 @@
           <t>BSMA0002</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>Not empirical (Qualitative study lacking quantitative correlations)</t>
@@ -872,11 +867,6 @@
       <c r="B12" t="inlineStr">
         <is>
           <t>BSMA0007</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">

</xml_diff>

<commit_message>
Auto-extracted measures for BSMA0001
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX12"/>
+  <dimension ref="A1:AX16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="12" min="1" max="2"/>
@@ -876,9 +876,51 @@
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="12"/>
-    <row r="14" ht="15.75" customHeight="1" s="12"/>
+    <row r="14" ht="15.75" customHeight="1" s="12">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>BSMA0001</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Not a quantitative empirical study (qualitative interviews with n=33 rural journalists, no correlation matrix) and not team-level.</t>
+        </is>
+      </c>
+    </row>
     <row r="15" ht="15.75" customHeight="1" s="12"/>
-    <row r="16" ht="15.75" customHeight="1" s="12"/>
+    <row r="16" ht="15.75" customHeight="1" s="12">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>BSMA0002</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>The paper is a qualitative study utilizing thematic analysis, not a quantitative empirical study, and does not contain a correlation matrix or measurable variables.</t>
+        </is>
+      </c>
+    </row>
     <row r="17" ht="15.75" customHeight="1" s="12"/>
     <row r="18" ht="15.75" customHeight="1" s="12"/>
     <row r="19" ht="15.75" customHeight="1" s="12"/>

</xml_diff>

<commit_message>
Auto-extracted measures for BSMA0003 (Excluded - File Not Found)
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX18"/>
+  <dimension ref="A1:AX20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="12" min="1" max="2"/>
@@ -945,7 +945,28 @@
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="12"/>
-    <row r="20" ht="15.75" customHeight="1" s="12"/>
+    <row r="20" ht="15.75" customHeight="1" s="12">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>BSMA0001</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Not a quantitative empirical study (qualitative interviews with n=33 rural journalists, no correlation matrix) and not team-level.</t>
+        </is>
+      </c>
+    </row>
     <row r="21" ht="15.75" customHeight="1" s="12"/>
     <row r="22" ht="15.75" customHeight="1" s="12"/>
     <row r="23" ht="15.75" customHeight="1" s="12"/>

</xml_diff>

<commit_message>
Auto-extracted measures for BSMA0003
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX24"/>
+  <dimension ref="A1:AX29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="12" min="1" max="2"/>
@@ -933,9 +933,19 @@
           <t>BSMA0003</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>BSMA0003.1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>BSMA0003.1.1</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
+          <t>1 = Include</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -943,8 +953,243 @@
           <t>File not found</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V18" t="n">
+        <v>192</v>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>Junior doctors and APNs</t>
+        </is>
+      </c>
+      <c r="AA18" t="n">
+        <v>999</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>999</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>999</v>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>An APN was present in 86 shifts.</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>0 = No APN, 1 = APN</t>
+        </is>
+      </c>
+      <c r="AH18" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK18" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM18" t="inlineStr">
+        <is>
+          <t>The average hospital experience of junior doctors.</t>
+        </is>
+      </c>
+      <c r="AN18" t="inlineStr">
+        <is>
+          <t>Years</t>
+        </is>
+      </c>
+      <c r="AO18" t="inlineStr">
+        <is>
+          <t>APN</t>
+        </is>
+      </c>
+      <c r="AP18" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="AQ18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AR18" t="n">
+        <v>999</v>
+      </c>
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t>Junior Doc. Experience</t>
+        </is>
+      </c>
+      <c r="AT18" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="AU18" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="AV18" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW18" t="n">
+        <v>-0.02</v>
+      </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1" s="12"/>
+    <row r="19" ht="15.75" customHeight="1" s="12">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>BSMA0003</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BSMA0003.1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>BSMA0003.1.2</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>File not found</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V19" t="n">
+        <v>192</v>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>Junior doctors and APNs</t>
+        </is>
+      </c>
+      <c r="AA19" t="n">
+        <v>999</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>999</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>999</v>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>An APN was present in 86 shifts.</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>0 = No APN, 1 = APN</t>
+        </is>
+      </c>
+      <c r="AH19" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK19" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM19" t="inlineStr">
+        <is>
+          <t>This information was taken from the pagers junior doctors carry on their overtime shift and recorded at the end of the shift.</t>
+        </is>
+      </c>
+      <c r="AN19" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="AO19" t="inlineStr">
+        <is>
+          <t>APN</t>
+        </is>
+      </c>
+      <c r="AP19" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="AQ19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AR19" t="n">
+        <v>999</v>
+      </c>
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t>Paged requests for assistance</t>
+        </is>
+      </c>
+      <c r="AT19" t="n">
+        <v>11.46</v>
+      </c>
+      <c r="AU19" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="AV19" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW19" t="n">
+        <v>-0.01</v>
+      </c>
+    </row>
     <row r="20" ht="15.75" customHeight="1" s="12">
       <c r="A20" t="inlineStr">
         <is>
@@ -953,21 +1198,266 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BSMA0001</t>
+          <t>BSMA0003</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BSMA0003.1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>BSMA0003.1.3</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
+          <t>1 = Include</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Not a quantitative empirical study (qualitative interviews with n=33 rural journalists, no correlation matrix) and not team-level.</t>
-        </is>
+          <t>File not found</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V20" t="n">
+        <v>192</v>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>Junior doctors and APNs</t>
+        </is>
+      </c>
+      <c r="AA20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>An APN was present in 86 shifts.</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>0 = No APN, 1 = APN</t>
+        </is>
+      </c>
+      <c r="AH20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK20" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM20" t="inlineStr">
+        <is>
+          <t>Junior doctors recorded their tasks and self-initiated ward rounds throughout the overtime shift and also noted the origin of the task, such as whether the task could have been completed during the day.</t>
+        </is>
+      </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="AO20" t="inlineStr">
+        <is>
+          <t>APN</t>
+        </is>
+      </c>
+      <c r="AP20" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="AQ20" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AR20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AS20" t="inlineStr">
+        <is>
+          <t>Tasks from day shift</t>
+        </is>
+      </c>
+      <c r="AT20" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="AU20" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="AV20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW20" t="n">
+        <v>-0.16</v>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1" s="12"/>
+    <row r="21" ht="15.75" customHeight="1" s="12">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>BSMA0003</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>BSMA0003.1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>BSMA0003.1.4</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>File not found</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V21" t="n">
+        <v>192</v>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>Junior doctors and APNs</t>
+        </is>
+      </c>
+      <c r="AA21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>An APN was present in 86 shifts.</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>0 = No APN, 1 = APN</t>
+        </is>
+      </c>
+      <c r="AH21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK21" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM21" t="inlineStr">
+        <is>
+          <t>Senior doctors and APNs also classified tasks into those that could be undertaken by junior doctors or skilled nurses (junior doctor/skilled nurse tasks) and tasks that could only be completed by junior doctors.</t>
+        </is>
+      </c>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="AO21" t="inlineStr">
+        <is>
+          <t>APN</t>
+        </is>
+      </c>
+      <c r="AP21" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="AQ21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AR21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AS21" t="inlineStr">
+        <is>
+          <t>Skilled nurse/doctor tasks</t>
+        </is>
+      </c>
+      <c r="AT21" t="n">
+        <v>5.68</v>
+      </c>
+      <c r="AU21" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="AV21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW21" t="n">
+        <v>-0.26</v>
+      </c>
+    </row>
     <row r="22" ht="15.75" customHeight="1" s="12">
       <c r="A22" t="inlineStr">
         <is>
@@ -976,48 +1466,335 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>BSMA0003</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>BSMA0003.1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>BSMA0003.1.5</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>File not found</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V22" t="n">
+        <v>192</v>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>Junior doctors and APNs</t>
+        </is>
+      </c>
+      <c r="AA22" t="n">
+        <v>999</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>999</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>999</v>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>An APN was present in 86 shifts.</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>0 = No APN, 1 = APN</t>
+        </is>
+      </c>
+      <c r="AH22" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI22" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ22" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK22" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM22" t="inlineStr">
+        <is>
+          <t>Finally 'total tasks' was based on all tasks the junior doctor recorded during overtime.</t>
+        </is>
+      </c>
+      <c r="AN22" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="AO22" t="inlineStr">
+        <is>
+          <t>APN</t>
+        </is>
+      </c>
+      <c r="AP22" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AR22" t="n">
+        <v>999</v>
+      </c>
+      <c r="AS22" t="inlineStr">
+        <is>
+          <t>Total tasks</t>
+        </is>
+      </c>
+      <c r="AT22" t="n">
+        <v>25.53</v>
+      </c>
+      <c r="AU22" t="n">
+        <v>13.03</v>
+      </c>
+      <c r="AV22" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW22" t="n">
+        <v>-0.16</v>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="12">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>BSMA0003</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>BSMA0003.1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>BSMA0003.1.6</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>File not found</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V23" t="n">
+        <v>192</v>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>Junior doctors and APNs</t>
+        </is>
+      </c>
+      <c r="AA23" t="n">
+        <v>999</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>999</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>999</v>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>An APN was present in 86 shifts.</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>0 = No APN, 1 = APN</t>
+        </is>
+      </c>
+      <c r="AH23" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI23" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ23" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK23" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM23" t="inlineStr">
+        <is>
+          <t>Junior doctors recorded their tasks and self-initiated ward rounds throughout the overtime shift...</t>
+        </is>
+      </c>
+      <c r="AN23" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="AO23" t="inlineStr">
+        <is>
+          <t>APN</t>
+        </is>
+      </c>
+      <c r="AP23" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="AQ23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AR23" t="n">
+        <v>999</v>
+      </c>
+      <c r="AS23" t="inlineStr">
+        <is>
+          <t>Self-initiated ward rounds</t>
+        </is>
+      </c>
+      <c r="AT23" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="AU23" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="AV23" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW23" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="12"/>
+    <row r="25" ht="15.75" customHeight="1" s="12">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>BSMA0001</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Not a quantitative empirical study (qualitative interviews with n=33 rural journalists, no correlation matrix) and not team-level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="12"/>
+    <row r="27" ht="15.75" customHeight="1" s="12">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
           <t>BSMA0006</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>File not found at specified location</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15.75" customHeight="1" s="12"/>
-    <row r="24" ht="15.75" customHeight="1" s="12">
-      <c r="A24" t="inlineStr">
+    <row r="28" ht="15.75" customHeight="1" s="12"/>
+    <row r="29" ht="15.75" customHeight="1" s="12">
+      <c r="A29" t="inlineStr">
         <is>
           <t>KY</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>BSMA0007</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>The boundary spanner is at the organizational level (inpatient psychiatric departments) rather than an individual employee.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15.75" customHeight="1" s="12"/>
-    <row r="26" ht="15.75" customHeight="1" s="12"/>
-    <row r="27" ht="15.75" customHeight="1" s="12"/>
-    <row r="28" ht="15.75" customHeight="1" s="12"/>
-    <row r="29" ht="15.75" customHeight="1" s="12"/>
     <row r="30" ht="15.75" customHeight="1" s="12"/>
     <row r="31" ht="15.75" customHeight="1" s="12"/>
     <row r="32" ht="15.75" customHeight="1" s="12"/>

</xml_diff>

<commit_message>
Auto-extracted measures for BSMA0008 Marrone et al. 2007
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX40"/>
+  <dimension ref="A1:AX45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="12" min="1" max="2"/>
@@ -1823,7 +1823,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG27" t="inlineStr"/>
       <c r="AH27" t="n">
         <v>11</v>
       </c>
@@ -1953,7 +1952,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG28" t="inlineStr"/>
       <c r="AH28" t="n">
         <v>999</v>
       </c>
@@ -2083,7 +2081,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG29" t="inlineStr"/>
       <c r="AH29" t="n">
         <v>999</v>
       </c>
@@ -2213,7 +2210,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG30" t="inlineStr"/>
       <c r="AH30" t="n">
         <v>17</v>
       </c>
@@ -2233,7 +2229,6 @@
           <t>Role stressors were indicated by expatriates (17 items; Rizzo et al., 1970; Beehr et al., 1976).</t>
         </is>
       </c>
-      <c r="AN30" t="inlineStr"/>
       <c r="AO30" t="inlineStr">
         <is>
           <t>Expatriates' boundary-spanning</t>
@@ -2339,7 +2334,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG31" t="inlineStr"/>
       <c r="AH31" t="n">
         <v>6</v>
       </c>
@@ -2359,7 +2353,6 @@
           <t>Subsidiary identification (reported by expatriates) and MNE identification (reported by host-country coworkers) were both measured using an organizational identification scale (six items; Mael &amp; Ashforth, 1992).</t>
         </is>
       </c>
-      <c r="AN31" t="inlineStr"/>
       <c r="AO31" t="inlineStr">
         <is>
           <t>Expatriates' boundary-spanning</t>
@@ -2465,7 +2458,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG32" t="inlineStr"/>
       <c r="AH32" t="n">
         <v>9</v>
       </c>
@@ -2485,7 +2477,6 @@
           <t>Emotional exhaustion was reported by expatriates (nine items; Maslach &amp; Jackson, 1981)</t>
         </is>
       </c>
-      <c r="AN32" t="inlineStr"/>
       <c r="AO32" t="inlineStr">
         <is>
           <t>Expatriates' boundary-spanning</t>
@@ -2591,7 +2582,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG33" t="inlineStr"/>
       <c r="AH33" t="n">
         <v>7</v>
       </c>
@@ -2611,7 +2601,6 @@
           <t>outgroup categorization was reported by host-country coworkers (seven items; Leonardelli &amp; Toh, 2011).</t>
         </is>
       </c>
-      <c r="AN33" t="inlineStr"/>
       <c r="AO33" t="inlineStr">
         <is>
           <t>Expatriates' boundary-spanning</t>
@@ -2717,7 +2706,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG34" t="inlineStr"/>
       <c r="AH34" t="n">
         <v>999</v>
       </c>
@@ -2847,7 +2835,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG35" t="inlineStr"/>
       <c r="AH35" t="n">
         <v>999</v>
       </c>
@@ -2977,7 +2964,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG36" t="inlineStr"/>
       <c r="AH36" t="n">
         <v>999</v>
       </c>
@@ -3107,7 +3093,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG37" t="inlineStr"/>
       <c r="AH37" t="n">
         <v>999</v>
       </c>
@@ -3237,7 +3222,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG38" t="inlineStr"/>
       <c r="AH38" t="n">
         <v>999</v>
       </c>
@@ -3317,11 +3301,619 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="15.75" customHeight="1" s="12"/>
-    <row r="42" ht="15.75" customHeight="1" s="12"/>
-    <row r="43" ht="15.75" customHeight="1" s="12"/>
-    <row r="44" ht="15.75" customHeight="1" s="12"/>
-    <row r="45" ht="15.75" customHeight="1" s="12"/>
+    <row r="41" ht="15.75" customHeight="1" s="12">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>BSMA0008</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>BSMA0008.1</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>BSMA0008.1.1</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V41" t="n">
+        <v>190</v>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>MBA students / Consulting</t>
+        </is>
+      </c>
+      <c r="AA41" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB41" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC41" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>3 = Others</t>
+        </is>
+      </c>
+      <c r="AF41" t="inlineStr">
+        <is>
+          <t>six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context.</t>
+        </is>
+      </c>
+      <c r="AG41" t="inlineStr"/>
+      <c r="AH41" t="n">
+        <v>6</v>
+      </c>
+      <c r="AI41" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ41" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK41" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM41" t="inlineStr">
+        <is>
+          <t>all participants rate the extent to which they perceived each of the six boundary spanning behaviors as an expected part of their responsibilities</t>
+        </is>
+      </c>
+      <c r="AN41" t="inlineStr"/>
+      <c r="AO41" t="inlineStr">
+        <is>
+          <t>Boundary-spanning behavior</t>
+        </is>
+      </c>
+      <c r="AP41" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="AQ41" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AR41" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AS41" t="inlineStr">
+        <is>
+          <t>Boundary-spanning role</t>
+        </is>
+      </c>
+      <c r="AT41" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="AU41" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="AV41" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AW41" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="42" ht="15.75" customHeight="1" s="12">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>BSMA0008</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>BSMA0008.1</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>BSMA0008.1.2</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V42" t="n">
+        <v>190</v>
+      </c>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>MBA students / Consulting</t>
+        </is>
+      </c>
+      <c r="AA42" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC42" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>3 = Others</t>
+        </is>
+      </c>
+      <c r="AF42" t="inlineStr">
+        <is>
+          <t>six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context.</t>
+        </is>
+      </c>
+      <c r="AG42" t="inlineStr"/>
+      <c r="AH42" t="n">
+        <v>8</v>
+      </c>
+      <c r="AI42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ42" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK42" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM42" t="inlineStr">
+        <is>
+          <t>Scale items were based in part upon Parker's (1998) role breadth self-efficacy scale</t>
+        </is>
+      </c>
+      <c r="AN42" t="inlineStr"/>
+      <c r="AO42" t="inlineStr">
+        <is>
+          <t>Boundary-spanning behavior</t>
+        </is>
+      </c>
+      <c r="AP42" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="AQ42" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AR42" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AS42" t="inlineStr">
+        <is>
+          <t>Boundary-spanning self-efficacy</t>
+        </is>
+      </c>
+      <c r="AT42" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="AU42" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="AV42" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="AW42" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1" s="12">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>BSMA0008</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>BSMA0008.1</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>BSMA0008.1.3</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V43" t="n">
+        <v>190</v>
+      </c>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>MBA students / Consulting</t>
+        </is>
+      </c>
+      <c r="AA43" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB43" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC43" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD43" t="inlineStr">
+        <is>
+          <t>3 = Others</t>
+        </is>
+      </c>
+      <c r="AF43" t="inlineStr">
+        <is>
+          <t>six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context.</t>
+        </is>
+      </c>
+      <c r="AG43" t="inlineStr"/>
+      <c r="AH43" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI43" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ43" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK43" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM43" t="inlineStr">
+        <is>
+          <t>Asian ethnicity (1, Asian, and 0, other)</t>
+        </is>
+      </c>
+      <c r="AN43" t="inlineStr">
+        <is>
+          <t>Demographic</t>
+        </is>
+      </c>
+      <c r="AO43" t="inlineStr">
+        <is>
+          <t>Boundary-spanning behavior</t>
+        </is>
+      </c>
+      <c r="AP43" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="AQ43" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AR43" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AS43" t="inlineStr">
+        <is>
+          <t>Asian ethnicity</t>
+        </is>
+      </c>
+      <c r="AT43" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="AU43" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="AV43" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW43" t="n">
+        <v>-0.23</v>
+      </c>
+    </row>
+    <row r="44" ht="15.75" customHeight="1" s="12">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>BSMA0008</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>BSMA0008.1</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>BSMA0008.1.4</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V44" t="n">
+        <v>190</v>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>MBA students / Consulting</t>
+        </is>
+      </c>
+      <c r="AA44" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB44" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC44" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD44" t="inlineStr">
+        <is>
+          <t>3 = Others</t>
+        </is>
+      </c>
+      <c r="AF44" t="inlineStr">
+        <is>
+          <t>six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context.</t>
+        </is>
+      </c>
+      <c r="AG44" t="inlineStr"/>
+      <c r="AH44" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI44" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ44" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK44" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM44" t="inlineStr">
+        <is>
+          <t>GMAT score (a continuous score)</t>
+        </is>
+      </c>
+      <c r="AN44" t="inlineStr">
+        <is>
+          <t>Proxy</t>
+        </is>
+      </c>
+      <c r="AO44" t="inlineStr">
+        <is>
+          <t>Boundary-spanning behavior</t>
+        </is>
+      </c>
+      <c r="AP44" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="AQ44" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AR44" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AS44" t="inlineStr">
+        <is>
+          <t>GMAT score</t>
+        </is>
+      </c>
+      <c r="AT44" t="n">
+        <v>653.9</v>
+      </c>
+      <c r="AU44" t="n">
+        <v>57.89</v>
+      </c>
+      <c r="AV44" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW44" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="45" ht="15.75" customHeight="1" s="12">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>BSMA0008</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>BSMA0008.1</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>BSMA0008.1.5</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V45" t="n">
+        <v>190</v>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>MBA students / Consulting</t>
+        </is>
+      </c>
+      <c r="AA45" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC45" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>3 = Others</t>
+        </is>
+      </c>
+      <c r="AF45" t="inlineStr">
+        <is>
+          <t>six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context.</t>
+        </is>
+      </c>
+      <c r="AG45" t="inlineStr"/>
+      <c r="AH45" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ45" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK45" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM45" t="inlineStr">
+        <is>
+          <t>Three items were adapted from Beehr et al. (1976) and modified for the current context.</t>
+        </is>
+      </c>
+      <c r="AN45" t="inlineStr"/>
+      <c r="AO45" t="inlineStr">
+        <is>
+          <t>Boundary-spanning behavior</t>
+        </is>
+      </c>
+      <c r="AP45" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="AQ45" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AR45" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AS45" t="inlineStr">
+        <is>
+          <t>Role overload</t>
+        </is>
+      </c>
+      <c r="AT45" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="AU45" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="AV45" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="AW45" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
     <row r="46" ht="15.75" customHeight="1" s="12"/>
     <row r="47" ht="15.75" customHeight="1" s="12"/>
     <row r="48" ht="15.75" customHeight="1" s="12"/>

</xml_diff>

<commit_message>
Deduplicate BSMA0006 rows caused by multiple retry injections
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX67"/>
+  <dimension ref="A1:AX45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="12" min="1" max="2"/>
@@ -1823,7 +1823,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG27" t="inlineStr"/>
       <c r="AH27" t="n">
         <v>11</v>
       </c>
@@ -1953,7 +1952,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG28" t="inlineStr"/>
       <c r="AH28" t="n">
         <v>999</v>
       </c>
@@ -2083,7 +2081,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG29" t="inlineStr"/>
       <c r="AH29" t="n">
         <v>999</v>
       </c>
@@ -2213,7 +2210,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG30" t="inlineStr"/>
       <c r="AH30" t="n">
         <v>17</v>
       </c>
@@ -2233,7 +2229,6 @@
           <t>Role stressors were indicated by expatriates (17 items; Rizzo et al., 1970; Beehr et al., 1976).</t>
         </is>
       </c>
-      <c r="AN30" t="inlineStr"/>
       <c r="AO30" t="inlineStr">
         <is>
           <t>Expatriates' boundary-spanning</t>
@@ -2339,7 +2334,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG31" t="inlineStr"/>
       <c r="AH31" t="n">
         <v>6</v>
       </c>
@@ -2359,7 +2353,6 @@
           <t>Subsidiary identification (reported by expatriates) and MNE identification (reported by host-country coworkers) were both measured using an organizational identification scale (six items; Mael &amp; Ashforth, 1992).</t>
         </is>
       </c>
-      <c r="AN31" t="inlineStr"/>
       <c r="AO31" t="inlineStr">
         <is>
           <t>Expatriates' boundary-spanning</t>
@@ -2465,7 +2458,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG32" t="inlineStr"/>
       <c r="AH32" t="n">
         <v>9</v>
       </c>
@@ -2485,7 +2477,6 @@
           <t>Emotional exhaustion was reported by expatriates (nine items; Maslach &amp; Jackson, 1981)</t>
         </is>
       </c>
-      <c r="AN32" t="inlineStr"/>
       <c r="AO32" t="inlineStr">
         <is>
           <t>Expatriates' boundary-spanning</t>
@@ -2591,7 +2582,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG33" t="inlineStr"/>
       <c r="AH33" t="n">
         <v>7</v>
       </c>
@@ -2611,7 +2601,6 @@
           <t>outgroup categorization was reported by host-country coworkers (seven items; Leonardelli &amp; Toh, 2011).</t>
         </is>
       </c>
-      <c r="AN33" t="inlineStr"/>
       <c r="AO33" t="inlineStr">
         <is>
           <t>Expatriates' boundary-spanning</t>
@@ -2717,7 +2706,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG34" t="inlineStr"/>
       <c r="AH34" t="n">
         <v>999</v>
       </c>
@@ -2847,7 +2835,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG35" t="inlineStr"/>
       <c r="AH35" t="n">
         <v>999</v>
       </c>
@@ -2977,7 +2964,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG36" t="inlineStr"/>
       <c r="AH36" t="n">
         <v>999</v>
       </c>
@@ -3107,7 +3093,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG37" t="inlineStr"/>
       <c r="AH37" t="n">
         <v>999</v>
       </c>
@@ -3237,7 +3222,6 @@
           <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
         </is>
       </c>
-      <c r="AG38" t="inlineStr"/>
       <c r="AH38" t="n">
         <v>999</v>
       </c>
@@ -3294,135 +3278,7 @@
         <v>-0.08</v>
       </c>
     </row>
-    <row r="39" ht="15.75" customHeight="1" s="12">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>BSMA0006.1</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>BSMA0006.1.2</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V39" t="n">
-        <v>177</v>
-      </c>
-      <c r="Z39" t="inlineStr">
-        <is>
-          <t>expatriates</t>
-        </is>
-      </c>
-      <c r="AA39" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB39" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC39" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD39" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AF39" t="inlineStr">
-        <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AH39" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI39" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ39" t="n">
-        <v>7</v>
-      </c>
-      <c r="AK39" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM39" t="inlineStr">
-        <is>
-          <t>Mutual trust, cognition-based mutual trust, and affect-based mutual trust were reported by both expatriates and host-country coworkers (11 items; McAllister, 1995).</t>
-        </is>
-      </c>
-      <c r="AN39" t="inlineStr">
-        <is>
-          <t>Reported by both expatriate and coworker.</t>
-        </is>
-      </c>
-      <c r="AO39" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AP39" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AQ39" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AR39" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AS39" t="inlineStr">
-        <is>
-          <t>Cognition-based mutual trust</t>
-        </is>
-      </c>
-      <c r="AT39" t="n">
-        <v>5.38</v>
-      </c>
-      <c r="AU39" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="AV39" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AW39" t="n">
-        <v>0.63</v>
-      </c>
-    </row>
+    <row r="39" ht="15.75" customHeight="1" s="12"/>
     <row r="40" ht="15.75" customHeight="1" s="12">
       <c r="A40" t="inlineStr">
         <is>
@@ -3431,125 +3287,18 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>BSMA0006.1</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>BSMA0006.1.3</t>
+          <t>BSMA0007</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>0 = Exclude</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q40" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U40" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V40" t="n">
-        <v>177</v>
-      </c>
-      <c r="Z40" t="inlineStr">
-        <is>
-          <t>expatriates</t>
-        </is>
-      </c>
-      <c r="AA40" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB40" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC40" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD40" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AF40" t="inlineStr">
-        <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AH40" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI40" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ40" t="n">
-        <v>7</v>
-      </c>
-      <c r="AK40" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM40" t="inlineStr">
-        <is>
-          <t>Mutual trust, cognition-based mutual trust, and affect-based mutual trust were reported by both expatriates and host-country coworkers (11 items; McAllister, 1995).</t>
-        </is>
-      </c>
-      <c r="AN40" t="inlineStr">
-        <is>
-          <t>Reported by both expatriate and coworker.</t>
-        </is>
-      </c>
-      <c r="AO40" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AP40" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AQ40" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AR40" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AS40" t="inlineStr">
-        <is>
-          <t>Affect-based mutual trust</t>
-        </is>
-      </c>
-      <c r="AT40" t="n">
-        <v>5.11</v>
-      </c>
-      <c r="AU40" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="AV40" t="n">
-        <v>0.87</v>
-      </c>
-      <c r="AW40" t="n">
-        <v>0.7</v>
+          <t>The boundary spanner is at the organizational level (inpatient psychiatric departments) rather than an individual employee.</t>
+        </is>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="12">
@@ -3560,17 +3309,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>BSMA0006</t>
+          <t>BSMA0008</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>BSMA0006.1</t>
+          <t>BSMA0008.1</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>BSMA0006.1.4</t>
+          <t>BSMA0008.1.1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3578,11 +3327,6 @@
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
       <c r="L41" t="inlineStr">
         <is>
           <t>1 = Journal article</t>
@@ -3599,40 +3343,40 @@
         </is>
       </c>
       <c r="V41" t="n">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="Z41" t="inlineStr">
         <is>
-          <t>expatriates</t>
+          <t>MBA students / Consulting</t>
         </is>
       </c>
       <c r="AA41" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="AB41" t="n">
         <v>1</v>
       </c>
       <c r="AC41" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AD41" t="inlineStr">
         <is>
-          <t>2 = Supervisor</t>
+          <t>3 = Others</t>
         </is>
       </c>
       <c r="AF41" t="inlineStr">
         <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
+          <t>six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context.</t>
         </is>
       </c>
       <c r="AH41" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="AI41" t="n">
         <v>1</v>
       </c>
       <c r="AJ41" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AK41" t="inlineStr">
         <is>
@@ -3641,39 +3385,39 @@
       </c>
       <c r="AM41" t="inlineStr">
         <is>
-          <t>Role stressors were indicated by expatriates (17 items; Rizzo et al., 1970; Beehr et al., 1976).</t>
+          <t>all participants rate the extent to which they perceived each of the six boundary spanning behaviors as an expected part of their responsibilities</t>
         </is>
       </c>
       <c r="AO41" t="inlineStr">
         <is>
-          <t>Expatriates' boundary-spanning</t>
+          <t>Boundary-spanning behavior</t>
         </is>
       </c>
       <c r="AP41" t="n">
-        <v>5.27</v>
+        <v>2.91</v>
       </c>
       <c r="AQ41" t="n">
-        <v>0.74</v>
+        <v>0.7</v>
       </c>
       <c r="AR41" t="n">
-        <v>0.96</v>
+        <v>0.86</v>
       </c>
       <c r="AS41" t="inlineStr">
         <is>
-          <t>Role stressors</t>
+          <t>Boundary-spanning role</t>
         </is>
       </c>
       <c r="AT41" t="n">
-        <v>3.64</v>
+        <v>3.09</v>
       </c>
       <c r="AU41" t="n">
-        <v>0.97</v>
+        <v>0.82</v>
       </c>
       <c r="AV41" t="n">
-        <v>0.93</v>
+        <v>0.86</v>
       </c>
       <c r="AW41" t="n">
-        <v>0.42</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="12">
@@ -3684,17 +3428,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>BSMA0006</t>
+          <t>BSMA0008</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>BSMA0006.1</t>
+          <t>BSMA0008.1</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>BSMA0006.1.5</t>
+          <t>BSMA0008.1.2</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3702,11 +3446,6 @@
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
       <c r="L42" t="inlineStr">
         <is>
           <t>1 = Journal article</t>
@@ -3723,40 +3462,40 @@
         </is>
       </c>
       <c r="V42" t="n">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="Z42" t="inlineStr">
         <is>
-          <t>expatriates</t>
+          <t>MBA students / Consulting</t>
         </is>
       </c>
       <c r="AA42" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="AB42" t="n">
         <v>1</v>
       </c>
       <c r="AC42" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AD42" t="inlineStr">
         <is>
-          <t>2 = Supervisor</t>
+          <t>3 = Others</t>
         </is>
       </c>
       <c r="AF42" t="inlineStr">
         <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
+          <t>six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context.</t>
         </is>
       </c>
       <c r="AH42" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AI42" t="n">
         <v>1</v>
       </c>
       <c r="AJ42" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AK42" t="inlineStr">
         <is>
@@ -3765,39 +3504,39 @@
       </c>
       <c r="AM42" t="inlineStr">
         <is>
-          <t>Subsidiary identification (reported by expatriates) and MNE identification (reported by host-country coworkers) were both measured using an organizational identification scale (six items; Mael &amp; Ashforth, 1992).</t>
+          <t>Scale items were based in part upon Parker's (1998) role breadth self-efficacy scale</t>
         </is>
       </c>
       <c r="AO42" t="inlineStr">
         <is>
-          <t>Expatriates' boundary-spanning</t>
+          <t>Boundary-spanning behavior</t>
         </is>
       </c>
       <c r="AP42" t="n">
-        <v>5.27</v>
+        <v>2.91</v>
       </c>
       <c r="AQ42" t="n">
-        <v>0.74</v>
+        <v>0.7</v>
       </c>
       <c r="AR42" t="n">
-        <v>0.96</v>
+        <v>0.86</v>
       </c>
       <c r="AS42" t="inlineStr">
         <is>
-          <t>Expatriates' subsidiary identification</t>
+          <t>Boundary-spanning self-efficacy</t>
         </is>
       </c>
       <c r="AT42" t="n">
-        <v>5.3</v>
+        <v>4.07</v>
       </c>
       <c r="AU42" t="n">
-        <v>0.95</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="AV42" t="n">
         <v>0.92</v>
       </c>
       <c r="AW42" t="n">
-        <v>0.45</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="12">
@@ -3808,17 +3547,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>BSMA0006</t>
+          <t>BSMA0008</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>BSMA0006.1</t>
+          <t>BSMA0008.1</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>BSMA0006.1.6</t>
+          <t>BSMA0008.1.3</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -3826,11 +3565,6 @@
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
       <c r="L43" t="inlineStr">
         <is>
           <t>1 = Journal article</t>
@@ -3847,40 +3581,40 @@
         </is>
       </c>
       <c r="V43" t="n">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="Z43" t="inlineStr">
         <is>
-          <t>expatriates</t>
+          <t>MBA students / Consulting</t>
         </is>
       </c>
       <c r="AA43" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="AB43" t="n">
         <v>1</v>
       </c>
       <c r="AC43" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AD43" t="inlineStr">
         <is>
-          <t>2 = Supervisor</t>
+          <t>3 = Others</t>
         </is>
       </c>
       <c r="AF43" t="inlineStr">
         <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
+          <t>six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context.</t>
         </is>
       </c>
       <c r="AH43" t="n">
-        <v>9</v>
+        <v>999</v>
       </c>
       <c r="AI43" t="n">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="AJ43" t="n">
-        <v>7</v>
+        <v>999</v>
       </c>
       <c r="AK43" t="inlineStr">
         <is>
@@ -3889,39 +3623,44 @@
       </c>
       <c r="AM43" t="inlineStr">
         <is>
-          <t>Emotional exhaustion was reported by expatriates (nine items; Maslach &amp; Jackson, 1981)</t>
+          <t>Asian ethnicity (1, Asian, and 0, other)</t>
+        </is>
+      </c>
+      <c r="AN43" t="inlineStr">
+        <is>
+          <t>Demographic</t>
         </is>
       </c>
       <c r="AO43" t="inlineStr">
         <is>
-          <t>Expatriates' boundary-spanning</t>
+          <t>Boundary-spanning behavior</t>
         </is>
       </c>
       <c r="AP43" t="n">
-        <v>5.27</v>
+        <v>2.91</v>
       </c>
       <c r="AQ43" t="n">
-        <v>0.74</v>
+        <v>0.7</v>
       </c>
       <c r="AR43" t="n">
-        <v>0.96</v>
+        <v>0.86</v>
       </c>
       <c r="AS43" t="inlineStr">
         <is>
-          <t>Expatriates' emotional exhaustion</t>
+          <t>Asian ethnicity</t>
         </is>
       </c>
       <c r="AT43" t="n">
-        <v>3.63</v>
+        <v>0.31</v>
       </c>
       <c r="AU43" t="n">
-        <v>1.49</v>
+        <v>0.46</v>
       </c>
       <c r="AV43" t="n">
-        <v>0.97</v>
+        <v>999</v>
       </c>
       <c r="AW43" t="n">
-        <v>-0.01</v>
+        <v>-0.23</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="12">
@@ -3932,17 +3671,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>BSMA0006</t>
+          <t>BSMA0008</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>BSMA0006.1</t>
+          <t>BSMA0008.1</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>BSMA0006.1.7</t>
+          <t>BSMA0008.1.4</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3950,11 +3689,6 @@
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
       <c r="L44" t="inlineStr">
         <is>
           <t>1 = Journal article</t>
@@ -3971,81 +3705,86 @@
         </is>
       </c>
       <c r="V44" t="n">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="Z44" t="inlineStr">
         <is>
-          <t>expatriates</t>
+          <t>MBA students / Consulting</t>
         </is>
       </c>
       <c r="AA44" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="AB44" t="n">
         <v>1</v>
       </c>
       <c r="AC44" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AD44" t="inlineStr">
         <is>
-          <t>2 = Supervisor</t>
+          <t>3 = Others</t>
         </is>
       </c>
       <c r="AF44" t="inlineStr">
         <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
+          <t>six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context.</t>
         </is>
       </c>
       <c r="AH44" t="n">
-        <v>7</v>
+        <v>999</v>
       </c>
       <c r="AI44" t="n">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="AJ44" t="n">
-        <v>7</v>
+        <v>999</v>
       </c>
       <c r="AK44" t="inlineStr">
         <is>
-          <t>2 = Supervisor</t>
+          <t>1 = Self</t>
         </is>
       </c>
       <c r="AM44" t="inlineStr">
         <is>
-          <t>outgroup categorization was reported by host-country coworkers (seven items; Leonardelli &amp; Toh, 2011).</t>
+          <t>GMAT score (a continuous score)</t>
+        </is>
+      </c>
+      <c r="AN44" t="inlineStr">
+        <is>
+          <t>Proxy</t>
         </is>
       </c>
       <c r="AO44" t="inlineStr">
         <is>
-          <t>Expatriates' boundary-spanning</t>
+          <t>Boundary-spanning behavior</t>
         </is>
       </c>
       <c r="AP44" t="n">
-        <v>5.27</v>
+        <v>2.91</v>
       </c>
       <c r="AQ44" t="n">
-        <v>0.74</v>
+        <v>0.7</v>
       </c>
       <c r="AR44" t="n">
-        <v>0.96</v>
+        <v>0.86</v>
       </c>
       <c r="AS44" t="inlineStr">
         <is>
-          <t>Expatriates' outgroup categorization</t>
+          <t>GMAT score</t>
         </is>
       </c>
       <c r="AT44" t="n">
-        <v>4.35</v>
+        <v>653.9</v>
       </c>
       <c r="AU44" t="n">
-        <v>0.97</v>
+        <v>57.89</v>
       </c>
       <c r="AV44" t="n">
-        <v>0.83</v>
+        <v>999</v>
       </c>
       <c r="AW44" t="n">
-        <v>0.25</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="12">
@@ -4056,17 +3795,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>BSMA0006</t>
+          <t>BSMA0008</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>BSMA0006.1</t>
+          <t>BSMA0008.1</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>BSMA0006.1.8</t>
+          <t>BSMA0008.1.5</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -4074,11 +3813,6 @@
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
       <c r="L45" t="inlineStr">
         <is>
           <t>1 = Journal article</t>
@@ -4095,40 +3829,40 @@
         </is>
       </c>
       <c r="V45" t="n">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="Z45" t="inlineStr">
         <is>
-          <t>expatriates</t>
+          <t>MBA students / Consulting</t>
         </is>
       </c>
       <c r="AA45" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="AB45" t="n">
         <v>1</v>
       </c>
       <c r="AC45" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AD45" t="inlineStr">
         <is>
-          <t>2 = Supervisor</t>
+          <t>3 = Others</t>
         </is>
       </c>
       <c r="AF45" t="inlineStr">
         <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
+          <t>six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context.</t>
         </is>
       </c>
       <c r="AH45" t="n">
-        <v>999</v>
+        <v>3</v>
       </c>
       <c r="AI45" t="n">
-        <v>999</v>
+        <v>1</v>
       </c>
       <c r="AJ45" t="n">
-        <v>999</v>
+        <v>5</v>
       </c>
       <c r="AK45" t="inlineStr">
         <is>
@@ -4137,2589 +3871,63 @@
       </c>
       <c r="AM45" t="inlineStr">
         <is>
-          <t>We included expatriates’ and host-country coworkers’ age, gender, industry, tenure in their subsidiaries, and foreign language proficiency (Liu &amp; Jackson, 2008).</t>
-        </is>
-      </c>
-      <c r="AN45" t="inlineStr">
-        <is>
-          <t>Years</t>
+          <t>Three items were adapted from Beehr et al. (1976) and modified for the current context.</t>
         </is>
       </c>
       <c r="AO45" t="inlineStr">
         <is>
-          <t>Expatriates' boundary-spanning</t>
+          <t>Boundary-spanning behavior</t>
         </is>
       </c>
       <c r="AP45" t="n">
-        <v>5.27</v>
+        <v>2.91</v>
       </c>
       <c r="AQ45" t="n">
-        <v>0.74</v>
+        <v>0.7</v>
       </c>
       <c r="AR45" t="n">
-        <v>0.96</v>
+        <v>0.86</v>
       </c>
       <c r="AS45" t="inlineStr">
         <is>
-          <t>Expatriate age</t>
+          <t>Role overload</t>
         </is>
       </c>
       <c r="AT45" t="n">
-        <v>33.91</v>
+        <v>2.47</v>
       </c>
       <c r="AU45" t="n">
-        <v>6.64</v>
+        <v>0.85</v>
       </c>
       <c r="AV45" t="n">
-        <v>999</v>
+        <v>0.83</v>
       </c>
       <c r="AW45" t="n">
-        <v>0.02</v>
+        <v>0.18</v>
       </c>
     </row>
-    <row r="46" ht="15.75" customHeight="1" s="12">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>BSMA0006.1</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>BSMA0006.1.9</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q46" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U46" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V46" t="n">
-        <v>177</v>
-      </c>
-      <c r="Z46" t="inlineStr">
-        <is>
-          <t>expatriates</t>
-        </is>
-      </c>
-      <c r="AA46" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB46" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC46" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD46" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AF46" t="inlineStr">
-        <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AH46" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI46" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ46" t="n">
-        <v>999</v>
-      </c>
-      <c r="AK46" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM46" t="inlineStr">
-        <is>
-          <t>We included expatriates’ and host-country coworkers’ age, gender, industry, tenure in their subsidiaries, and foreign language proficiency (Liu &amp; Jackson, 2008).</t>
-        </is>
-      </c>
-      <c r="AN46" t="inlineStr">
-        <is>
-          <t>1 = male, 2 = female</t>
-        </is>
-      </c>
-      <c r="AO46" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AP46" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AQ46" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AR46" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AS46" t="inlineStr">
-        <is>
-          <t>Expatriate gender</t>
-        </is>
-      </c>
-      <c r="AT46" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="AU46" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AV46" t="n">
-        <v>999</v>
-      </c>
-      <c r="AW46" t="n">
-        <v>-0.06</v>
-      </c>
-    </row>
-    <row r="47" ht="15.75" customHeight="1" s="12">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>BSMA0006.1</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>BSMA0006.1.10</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U47" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V47" t="n">
-        <v>177</v>
-      </c>
-      <c r="Z47" t="inlineStr">
-        <is>
-          <t>expatriates</t>
-        </is>
-      </c>
-      <c r="AA47" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB47" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC47" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD47" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AF47" t="inlineStr">
-        <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AH47" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI47" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ47" t="n">
-        <v>999</v>
-      </c>
-      <c r="AK47" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM47" t="inlineStr">
-        <is>
-          <t>We included expatriates’ and host-country coworkers’ age, gender, industry, tenure in their subsidiaries, and foreign language proficiency (Liu &amp; Jackson, 2008).</t>
-        </is>
-      </c>
-      <c r="AN47" t="inlineStr">
-        <is>
-          <t>Years</t>
-        </is>
-      </c>
-      <c r="AO47" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AP47" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AQ47" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AR47" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AS47" t="inlineStr">
-        <is>
-          <t>Expatriate tenure</t>
-        </is>
-      </c>
-      <c r="AT47" t="n">
-        <v>2.63</v>
-      </c>
-      <c r="AU47" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="AV47" t="n">
-        <v>999</v>
-      </c>
-      <c r="AW47" t="n">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="48" ht="15.75" customHeight="1" s="12">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>BSMA0006.1</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>BSMA0006.1.11</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q48" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U48" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V48" t="n">
-        <v>177</v>
-      </c>
-      <c r="Z48" t="inlineStr">
-        <is>
-          <t>expatriates</t>
-        </is>
-      </c>
-      <c r="AA48" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB48" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC48" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD48" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AF48" t="inlineStr">
-        <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AH48" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI48" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ48" t="n">
-        <v>999</v>
-      </c>
-      <c r="AK48" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM48" t="inlineStr">
-        <is>
-          <t>We included expatriates’ and host-country coworkers’ age, gender, industry, tenure in their subsidiaries, and foreign language proficiency (Liu &amp; Jackson, 2008).</t>
-        </is>
-      </c>
-      <c r="AN48" t="inlineStr">
-        <is>
-          <t>Proxy for language proficiency.</t>
-        </is>
-      </c>
-      <c r="AO48" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AP48" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AQ48" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AR48" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AS48" t="inlineStr">
-        <is>
-          <t>Expatriate language proficiency</t>
-        </is>
-      </c>
-      <c r="AT48" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="AU48" t="n">
-        <v>1.46</v>
-      </c>
-      <c r="AV48" t="n">
-        <v>999</v>
-      </c>
-      <c r="AW48" t="n">
-        <v>0.47</v>
-      </c>
-    </row>
-    <row r="49" ht="15.75" customHeight="1" s="12">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>BSMA0006.1</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>BSMA0006.1.12</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U49" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V49" t="n">
-        <v>177</v>
-      </c>
-      <c r="Z49" t="inlineStr">
-        <is>
-          <t>expatriates</t>
-        </is>
-      </c>
-      <c r="AA49" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB49" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC49" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD49" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AF49" t="inlineStr">
-        <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AH49" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI49" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ49" t="n">
-        <v>999</v>
-      </c>
-      <c r="AK49" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM49" t="inlineStr">
-        <is>
-          <t>We included expatriates’ and host-country coworkers’ age, gender, industry, tenure in their subsidiaries, and foreign language proficiency (Liu &amp; Jackson, 2008).</t>
-        </is>
-      </c>
-      <c r="AN49" t="inlineStr">
-        <is>
-          <t>Dummy control variable.</t>
-        </is>
-      </c>
-      <c r="AO49" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AP49" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AQ49" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AR49" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AS49" t="inlineStr">
-        <is>
-          <t>Industry</t>
-        </is>
-      </c>
-      <c r="AT49" t="n">
-        <v>5.7</v>
-      </c>
-      <c r="AU49" t="n">
-        <v>2.82</v>
-      </c>
-      <c r="AV49" t="n">
-        <v>999</v>
-      </c>
-      <c r="AW49" t="n">
-        <v>-0.08</v>
-      </c>
-    </row>
-    <row r="50" ht="15.75" customHeight="1" s="12">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>BSMA0006.1</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>BSMA0006.1.2</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q50" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U50" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V50" t="n">
-        <v>177</v>
-      </c>
-      <c r="Z50" t="inlineStr">
-        <is>
-          <t>expatriates</t>
-        </is>
-      </c>
-      <c r="AA50" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB50" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC50" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD50" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AF50" t="inlineStr">
-        <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AH50" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI50" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ50" t="n">
-        <v>7</v>
-      </c>
-      <c r="AK50" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM50" t="inlineStr">
-        <is>
-          <t>Mutual trust, cognition-based mutual trust, and affect-based mutual trust were reported by both expatriates and host-country coworkers (11 items; McAllister, 1995).</t>
-        </is>
-      </c>
-      <c r="AN50" t="inlineStr">
-        <is>
-          <t>Reported by both expatriate and coworker.</t>
-        </is>
-      </c>
-      <c r="AO50" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AP50" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AQ50" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AR50" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AS50" t="inlineStr">
-        <is>
-          <t>Cognition-based mutual trust</t>
-        </is>
-      </c>
-      <c r="AT50" t="n">
-        <v>5.38</v>
-      </c>
-      <c r="AU50" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="AV50" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AW50" t="n">
-        <v>0.63</v>
-      </c>
-    </row>
-    <row r="51" ht="15.75" customHeight="1" s="12">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>BSMA0006.1</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>BSMA0006.1.3</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U51" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V51" t="n">
-        <v>177</v>
-      </c>
-      <c r="Z51" t="inlineStr">
-        <is>
-          <t>expatriates</t>
-        </is>
-      </c>
-      <c r="AA51" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB51" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC51" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD51" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AF51" t="inlineStr">
-        <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AH51" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI51" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ51" t="n">
-        <v>7</v>
-      </c>
-      <c r="AK51" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM51" t="inlineStr">
-        <is>
-          <t>Mutual trust, cognition-based mutual trust, and affect-based mutual trust were reported by both expatriates and host-country coworkers (11 items; McAllister, 1995).</t>
-        </is>
-      </c>
-      <c r="AN51" t="inlineStr">
-        <is>
-          <t>Reported by both expatriate and coworker.</t>
-        </is>
-      </c>
-      <c r="AO51" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AP51" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AQ51" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AR51" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AS51" t="inlineStr">
-        <is>
-          <t>Affect-based mutual trust</t>
-        </is>
-      </c>
-      <c r="AT51" t="n">
-        <v>5.11</v>
-      </c>
-      <c r="AU51" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="AV51" t="n">
-        <v>0.87</v>
-      </c>
-      <c r="AW51" t="n">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="52" ht="15.75" customHeight="1" s="12">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>BSMA0006.1</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>BSMA0006.1.4</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q52" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U52" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V52" t="n">
-        <v>177</v>
-      </c>
-      <c r="Z52" t="inlineStr">
-        <is>
-          <t>expatriates</t>
-        </is>
-      </c>
-      <c r="AA52" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB52" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC52" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD52" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AF52" t="inlineStr">
-        <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AH52" t="n">
-        <v>17</v>
-      </c>
-      <c r="AI52" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ52" t="n">
-        <v>7</v>
-      </c>
-      <c r="AK52" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM52" t="inlineStr">
-        <is>
-          <t>Role stressors were indicated by expatriates (17 items; Rizzo et al., 1970; Beehr et al., 1976).</t>
-        </is>
-      </c>
-      <c r="AO52" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AP52" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AQ52" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AR52" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AS52" t="inlineStr">
-        <is>
-          <t>Role stressors</t>
-        </is>
-      </c>
-      <c r="AT52" t="n">
-        <v>3.64</v>
-      </c>
-      <c r="AU52" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="AV52" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="AW52" t="n">
-        <v>0.42</v>
-      </c>
-    </row>
-    <row r="53" ht="15.75" customHeight="1" s="12">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>BSMA0006.1</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>BSMA0006.1.5</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q53" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U53" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V53" t="n">
-        <v>177</v>
-      </c>
-      <c r="Z53" t="inlineStr">
-        <is>
-          <t>expatriates</t>
-        </is>
-      </c>
-      <c r="AA53" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB53" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC53" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD53" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AF53" t="inlineStr">
-        <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AH53" t="n">
-        <v>6</v>
-      </c>
-      <c r="AI53" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ53" t="n">
-        <v>7</v>
-      </c>
-      <c r="AK53" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM53" t="inlineStr">
-        <is>
-          <t>Subsidiary identification (reported by expatriates) and MNE identification (reported by host-country coworkers) were both measured using an organizational identification scale (six items; Mael &amp; Ashforth, 1992).</t>
-        </is>
-      </c>
-      <c r="AO53" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AP53" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AQ53" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AR53" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AS53" t="inlineStr">
-        <is>
-          <t>Expatriates' subsidiary identification</t>
-        </is>
-      </c>
-      <c r="AT53" t="n">
-        <v>5.3</v>
-      </c>
-      <c r="AU53" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="AV53" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="AW53" t="n">
-        <v>0.45</v>
-      </c>
-    </row>
-    <row r="54" ht="15.75" customHeight="1" s="12">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>BSMA0006.1</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>BSMA0006.1.6</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q54" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U54" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V54" t="n">
-        <v>177</v>
-      </c>
-      <c r="Z54" t="inlineStr">
-        <is>
-          <t>expatriates</t>
-        </is>
-      </c>
-      <c r="AA54" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB54" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC54" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD54" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AF54" t="inlineStr">
-        <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AH54" t="n">
-        <v>9</v>
-      </c>
-      <c r="AI54" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ54" t="n">
-        <v>7</v>
-      </c>
-      <c r="AK54" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM54" t="inlineStr">
-        <is>
-          <t>Emotional exhaustion was reported by expatriates (nine items; Maslach &amp; Jackson, 1981)</t>
-        </is>
-      </c>
-      <c r="AO54" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AP54" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AQ54" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AR54" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AS54" t="inlineStr">
-        <is>
-          <t>Expatriates' emotional exhaustion</t>
-        </is>
-      </c>
-      <c r="AT54" t="n">
-        <v>3.63</v>
-      </c>
-      <c r="AU54" t="n">
-        <v>1.49</v>
-      </c>
-      <c r="AV54" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="AW54" t="n">
-        <v>-0.01</v>
-      </c>
-    </row>
-    <row r="55" ht="15.75" customHeight="1" s="12">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>BSMA0006.1</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>BSMA0006.1.7</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q55" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U55" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V55" t="n">
-        <v>177</v>
-      </c>
-      <c r="Z55" t="inlineStr">
-        <is>
-          <t>expatriates</t>
-        </is>
-      </c>
-      <c r="AA55" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB55" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC55" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD55" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AF55" t="inlineStr">
-        <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AH55" t="n">
-        <v>7</v>
-      </c>
-      <c r="AI55" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ55" t="n">
-        <v>7</v>
-      </c>
-      <c r="AK55" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AM55" t="inlineStr">
-        <is>
-          <t>outgroup categorization was reported by host-country coworkers (seven items; Leonardelli &amp; Toh, 2011).</t>
-        </is>
-      </c>
-      <c r="AO55" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AP55" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AQ55" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AR55" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AS55" t="inlineStr">
-        <is>
-          <t>Expatriates' outgroup categorization</t>
-        </is>
-      </c>
-      <c r="AT55" t="n">
-        <v>4.35</v>
-      </c>
-      <c r="AU55" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="AV55" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="AW55" t="n">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="56" ht="15.75" customHeight="1" s="12">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>BSMA0006.1</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>BSMA0006.1.8</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q56" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U56" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V56" t="n">
-        <v>177</v>
-      </c>
-      <c r="Z56" t="inlineStr">
-        <is>
-          <t>expatriates</t>
-        </is>
-      </c>
-      <c r="AA56" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB56" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC56" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD56" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AF56" t="inlineStr">
-        <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AH56" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI56" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ56" t="n">
-        <v>999</v>
-      </c>
-      <c r="AK56" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM56" t="inlineStr">
-        <is>
-          <t>We included expatriates’ and host-country coworkers’ age, gender, industry, tenure in their subsidiaries, and foreign language proficiency (Liu &amp; Jackson, 2008).</t>
-        </is>
-      </c>
-      <c r="AN56" t="inlineStr">
-        <is>
-          <t>Years</t>
-        </is>
-      </c>
-      <c r="AO56" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AP56" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AQ56" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AR56" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AS56" t="inlineStr">
-        <is>
-          <t>Expatriate age</t>
-        </is>
-      </c>
-      <c r="AT56" t="n">
-        <v>33.91</v>
-      </c>
-      <c r="AU56" t="n">
-        <v>6.64</v>
-      </c>
-      <c r="AV56" t="n">
-        <v>999</v>
-      </c>
-      <c r="AW56" t="n">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="57" ht="15.75" customHeight="1" s="12">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>BSMA0006.1</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>BSMA0006.1.9</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q57" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U57" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V57" t="n">
-        <v>177</v>
-      </c>
-      <c r="Z57" t="inlineStr">
-        <is>
-          <t>expatriates</t>
-        </is>
-      </c>
-      <c r="AA57" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB57" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC57" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD57" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AF57" t="inlineStr">
-        <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AH57" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI57" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ57" t="n">
-        <v>999</v>
-      </c>
-      <c r="AK57" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM57" t="inlineStr">
-        <is>
-          <t>We included expatriates’ and host-country coworkers’ age, gender, industry, tenure in their subsidiaries, and foreign language proficiency (Liu &amp; Jackson, 2008).</t>
-        </is>
-      </c>
-      <c r="AN57" t="inlineStr">
-        <is>
-          <t>1 = male, 2 = female</t>
-        </is>
-      </c>
-      <c r="AO57" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AP57" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AQ57" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AR57" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AS57" t="inlineStr">
-        <is>
-          <t>Expatriate gender</t>
-        </is>
-      </c>
-      <c r="AT57" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="AU57" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AV57" t="n">
-        <v>999</v>
-      </c>
-      <c r="AW57" t="n">
-        <v>-0.06</v>
-      </c>
-    </row>
-    <row r="58" ht="15.75" customHeight="1" s="12">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>BSMA0006.1</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>BSMA0006.1.10</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q58" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U58" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V58" t="n">
-        <v>177</v>
-      </c>
-      <c r="Z58" t="inlineStr">
-        <is>
-          <t>expatriates</t>
-        </is>
-      </c>
-      <c r="AA58" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB58" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC58" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD58" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AF58" t="inlineStr">
-        <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AH58" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI58" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ58" t="n">
-        <v>999</v>
-      </c>
-      <c r="AK58" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM58" t="inlineStr">
-        <is>
-          <t>We included expatriates’ and host-country coworkers’ age, gender, industry, tenure in their subsidiaries, and foreign language proficiency (Liu &amp; Jackson, 2008).</t>
-        </is>
-      </c>
-      <c r="AN58" t="inlineStr">
-        <is>
-          <t>Years</t>
-        </is>
-      </c>
-      <c r="AO58" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AP58" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AQ58" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AR58" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AS58" t="inlineStr">
-        <is>
-          <t>Expatriate tenure</t>
-        </is>
-      </c>
-      <c r="AT58" t="n">
-        <v>2.63</v>
-      </c>
-      <c r="AU58" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="AV58" t="n">
-        <v>999</v>
-      </c>
-      <c r="AW58" t="n">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="59" ht="15.75" customHeight="1" s="12">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>BSMA0006.1</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>BSMA0006.1.11</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q59" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U59" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V59" t="n">
-        <v>177</v>
-      </c>
-      <c r="Z59" t="inlineStr">
-        <is>
-          <t>expatriates</t>
-        </is>
-      </c>
-      <c r="AA59" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB59" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC59" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD59" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AF59" t="inlineStr">
-        <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AH59" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI59" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ59" t="n">
-        <v>999</v>
-      </c>
-      <c r="AK59" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM59" t="inlineStr">
-        <is>
-          <t>We included expatriates’ and host-country coworkers’ age, gender, industry, tenure in their subsidiaries, and foreign language proficiency (Liu &amp; Jackson, 2008).</t>
-        </is>
-      </c>
-      <c r="AN59" t="inlineStr">
-        <is>
-          <t>Proxy for language proficiency.</t>
-        </is>
-      </c>
-      <c r="AO59" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AP59" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AQ59" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AR59" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AS59" t="inlineStr">
-        <is>
-          <t>Expatriate language proficiency</t>
-        </is>
-      </c>
-      <c r="AT59" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="AU59" t="n">
-        <v>1.46</v>
-      </c>
-      <c r="AV59" t="n">
-        <v>999</v>
-      </c>
-      <c r="AW59" t="n">
-        <v>0.47</v>
-      </c>
-    </row>
-    <row r="60" ht="15.75" customHeight="1" s="12">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>BSMA0006</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>BSMA0006.1</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>BSMA0006.1.12</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>File not found at specified location</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q60" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U60" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V60" t="n">
-        <v>177</v>
-      </c>
-      <c r="Z60" t="inlineStr">
-        <is>
-          <t>expatriates</t>
-        </is>
-      </c>
-      <c r="AA60" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB60" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC60" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD60" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AF60" t="inlineStr">
-        <is>
-          <t>We developed a new scale for expatriates’ boundary-spanning following Hinkin’s (1998) scale-development procedure. ... our final 26-item scale includes nine items for functional, seven items for linguistic, and ten items for cultural boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AH60" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI60" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ60" t="n">
-        <v>999</v>
-      </c>
-      <c r="AK60" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM60" t="inlineStr">
-        <is>
-          <t>We included expatriates’ and host-country coworkers’ age, gender, industry, tenure in their subsidiaries, and foreign language proficiency (Liu &amp; Jackson, 2008).</t>
-        </is>
-      </c>
-      <c r="AN60" t="inlineStr">
-        <is>
-          <t>Dummy control variable.</t>
-        </is>
-      </c>
-      <c r="AO60" t="inlineStr">
-        <is>
-          <t>Expatriates' boundary-spanning</t>
-        </is>
-      </c>
-      <c r="AP60" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="AQ60" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="AR60" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="AS60" t="inlineStr">
-        <is>
-          <t>Industry</t>
-        </is>
-      </c>
-      <c r="AT60" t="n">
-        <v>5.7</v>
-      </c>
-      <c r="AU60" t="n">
-        <v>2.82</v>
-      </c>
-      <c r="AV60" t="n">
-        <v>999</v>
-      </c>
-      <c r="AW60" t="n">
-        <v>-0.08</v>
-      </c>
-    </row>
+    <row r="46" ht="15.75" customHeight="1" s="12"/>
+    <row r="47" ht="15.75" customHeight="1" s="12"/>
+    <row r="48" ht="15.75" customHeight="1" s="12"/>
+    <row r="49" ht="15.75" customHeight="1" s="12"/>
+    <row r="50" ht="15.75" customHeight="1" s="12"/>
+    <row r="51" ht="15.75" customHeight="1" s="12"/>
+    <row r="52" ht="15.75" customHeight="1" s="12"/>
+    <row r="53" ht="15.75" customHeight="1" s="12"/>
+    <row r="54" ht="15.75" customHeight="1" s="12"/>
+    <row r="55" ht="15.75" customHeight="1" s="12"/>
+    <row r="56" ht="15.75" customHeight="1" s="12"/>
+    <row r="57" ht="15.75" customHeight="1" s="12"/>
+    <row r="58" ht="15.75" customHeight="1" s="12"/>
+    <row r="59" ht="15.75" customHeight="1" s="12"/>
+    <row r="60" ht="15.75" customHeight="1" s="12"/>
     <row r="61" ht="15.75" customHeight="1" s="12"/>
-    <row r="62" ht="15.75" customHeight="1" s="12">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>BSMA0007</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>The boundary spanner is at the organizational level (inpatient psychiatric departments) rather than an individual employee.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="15.75" customHeight="1" s="12">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>BSMA0008</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>BSMA0008.1</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>BSMA0008.1.1</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q63" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U63" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V63" t="n">
-        <v>190</v>
-      </c>
-      <c r="Z63" t="inlineStr">
-        <is>
-          <t>MBA students / Consulting</t>
-        </is>
-      </c>
-      <c r="AA63" t="n">
-        <v>6</v>
-      </c>
-      <c r="AB63" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC63" t="n">
-        <v>5</v>
-      </c>
-      <c r="AD63" t="inlineStr">
-        <is>
-          <t>3 = Others</t>
-        </is>
-      </c>
-      <c r="AF63" t="inlineStr">
-        <is>
-          <t>six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context.</t>
-        </is>
-      </c>
-      <c r="AH63" t="n">
-        <v>6</v>
-      </c>
-      <c r="AI63" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ63" t="n">
-        <v>5</v>
-      </c>
-      <c r="AK63" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM63" t="inlineStr">
-        <is>
-          <t>all participants rate the extent to which they perceived each of the six boundary spanning behaviors as an expected part of their responsibilities</t>
-        </is>
-      </c>
-      <c r="AO63" t="inlineStr">
-        <is>
-          <t>Boundary-spanning behavior</t>
-        </is>
-      </c>
-      <c r="AP63" t="n">
-        <v>2.91</v>
-      </c>
-      <c r="AQ63" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AR63" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="AS63" t="inlineStr">
-        <is>
-          <t>Boundary-spanning role</t>
-        </is>
-      </c>
-      <c r="AT63" t="n">
-        <v>3.09</v>
-      </c>
-      <c r="AU63" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="AV63" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="AW63" t="n">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="64" ht="15.75" customHeight="1" s="12">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>BSMA0008</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>BSMA0008.1</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>BSMA0008.1.2</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q64" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U64" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V64" t="n">
-        <v>190</v>
-      </c>
-      <c r="Z64" t="inlineStr">
-        <is>
-          <t>MBA students / Consulting</t>
-        </is>
-      </c>
-      <c r="AA64" t="n">
-        <v>6</v>
-      </c>
-      <c r="AB64" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC64" t="n">
-        <v>5</v>
-      </c>
-      <c r="AD64" t="inlineStr">
-        <is>
-          <t>3 = Others</t>
-        </is>
-      </c>
-      <c r="AF64" t="inlineStr">
-        <is>
-          <t>six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context.</t>
-        </is>
-      </c>
-      <c r="AH64" t="n">
-        <v>8</v>
-      </c>
-      <c r="AI64" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ64" t="n">
-        <v>5</v>
-      </c>
-      <c r="AK64" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM64" t="inlineStr">
-        <is>
-          <t>Scale items were based in part upon Parker's (1998) role breadth self-efficacy scale</t>
-        </is>
-      </c>
-      <c r="AO64" t="inlineStr">
-        <is>
-          <t>Boundary-spanning behavior</t>
-        </is>
-      </c>
-      <c r="AP64" t="n">
-        <v>2.91</v>
-      </c>
-      <c r="AQ64" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AR64" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="AS64" t="inlineStr">
-        <is>
-          <t>Boundary-spanning self-efficacy</t>
-        </is>
-      </c>
-      <c r="AT64" t="n">
-        <v>4.07</v>
-      </c>
-      <c r="AU64" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="AV64" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="AW64" t="n">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="65" ht="15.75" customHeight="1" s="12">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>BSMA0008</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>BSMA0008.1</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>BSMA0008.1.3</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q65" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U65" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V65" t="n">
-        <v>190</v>
-      </c>
-      <c r="Z65" t="inlineStr">
-        <is>
-          <t>MBA students / Consulting</t>
-        </is>
-      </c>
-      <c r="AA65" t="n">
-        <v>6</v>
-      </c>
-      <c r="AB65" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC65" t="n">
-        <v>5</v>
-      </c>
-      <c r="AD65" t="inlineStr">
-        <is>
-          <t>3 = Others</t>
-        </is>
-      </c>
-      <c r="AF65" t="inlineStr">
-        <is>
-          <t>six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context.</t>
-        </is>
-      </c>
-      <c r="AH65" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI65" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ65" t="n">
-        <v>999</v>
-      </c>
-      <c r="AK65" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM65" t="inlineStr">
-        <is>
-          <t>Asian ethnicity (1, Asian, and 0, other)</t>
-        </is>
-      </c>
-      <c r="AN65" t="inlineStr">
-        <is>
-          <t>Demographic</t>
-        </is>
-      </c>
-      <c r="AO65" t="inlineStr">
-        <is>
-          <t>Boundary-spanning behavior</t>
-        </is>
-      </c>
-      <c r="AP65" t="n">
-        <v>2.91</v>
-      </c>
-      <c r="AQ65" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AR65" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="AS65" t="inlineStr">
-        <is>
-          <t>Asian ethnicity</t>
-        </is>
-      </c>
-      <c r="AT65" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="AU65" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="AV65" t="n">
-        <v>999</v>
-      </c>
-      <c r="AW65" t="n">
-        <v>-0.23</v>
-      </c>
-    </row>
-    <row r="66" ht="15.75" customHeight="1" s="12">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>BSMA0008</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>BSMA0008.1</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>BSMA0008.1.4</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="L66" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q66" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U66" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V66" t="n">
-        <v>190</v>
-      </c>
-      <c r="Z66" t="inlineStr">
-        <is>
-          <t>MBA students / Consulting</t>
-        </is>
-      </c>
-      <c r="AA66" t="n">
-        <v>6</v>
-      </c>
-      <c r="AB66" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC66" t="n">
-        <v>5</v>
-      </c>
-      <c r="AD66" t="inlineStr">
-        <is>
-          <t>3 = Others</t>
-        </is>
-      </c>
-      <c r="AF66" t="inlineStr">
-        <is>
-          <t>six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context.</t>
-        </is>
-      </c>
-      <c r="AH66" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI66" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ66" t="n">
-        <v>999</v>
-      </c>
-      <c r="AK66" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM66" t="inlineStr">
-        <is>
-          <t>GMAT score (a continuous score)</t>
-        </is>
-      </c>
-      <c r="AN66" t="inlineStr">
-        <is>
-          <t>Proxy</t>
-        </is>
-      </c>
-      <c r="AO66" t="inlineStr">
-        <is>
-          <t>Boundary-spanning behavior</t>
-        </is>
-      </c>
-      <c r="AP66" t="n">
-        <v>2.91</v>
-      </c>
-      <c r="AQ66" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AR66" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="AS66" t="inlineStr">
-        <is>
-          <t>GMAT score</t>
-        </is>
-      </c>
-      <c r="AT66" t="n">
-        <v>653.9</v>
-      </c>
-      <c r="AU66" t="n">
-        <v>57.89</v>
-      </c>
-      <c r="AV66" t="n">
-        <v>999</v>
-      </c>
-      <c r="AW66" t="n">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="67" ht="15.75" customHeight="1" s="12">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>BSMA0008</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>BSMA0008.1</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>BSMA0008.1.5</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q67" t="inlineStr">
-        <is>
-          <t>1 = Cross-sectional</t>
-        </is>
-      </c>
-      <c r="U67" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V67" t="n">
-        <v>190</v>
-      </c>
-      <c r="Z67" t="inlineStr">
-        <is>
-          <t>MBA students / Consulting</t>
-        </is>
-      </c>
-      <c r="AA67" t="n">
-        <v>6</v>
-      </c>
-      <c r="AB67" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC67" t="n">
-        <v>5</v>
-      </c>
-      <c r="AD67" t="inlineStr">
-        <is>
-          <t>3 = Others</t>
-        </is>
-      </c>
-      <c r="AF67" t="inlineStr">
-        <is>
-          <t>six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context.</t>
-        </is>
-      </c>
-      <c r="AH67" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI67" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ67" t="n">
-        <v>5</v>
-      </c>
-      <c r="AK67" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM67" t="inlineStr">
-        <is>
-          <t>Three items were adapted from Beehr et al. (1976) and modified for the current context.</t>
-        </is>
-      </c>
-      <c r="AO67" t="inlineStr">
-        <is>
-          <t>Boundary-spanning behavior</t>
-        </is>
-      </c>
-      <c r="AP67" t="n">
-        <v>2.91</v>
-      </c>
-      <c r="AQ67" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AR67" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="AS67" t="inlineStr">
-        <is>
-          <t>Role overload</t>
-        </is>
-      </c>
-      <c r="AT67" t="n">
-        <v>2.47</v>
-      </c>
-      <c r="AU67" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="AV67" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="AW67" t="n">
-        <v>0.18</v>
-      </c>
-    </row>
+    <row r="62" ht="15.75" customHeight="1" s="12"/>
+    <row r="63" ht="15.75" customHeight="1" s="12"/>
+    <row r="64" ht="15.75" customHeight="1" s="12"/>
+    <row r="65" ht="15.75" customHeight="1" s="12"/>
+    <row r="66" ht="15.75" customHeight="1" s="12"/>
+    <row r="67" ht="15.75" customHeight="1" s="12"/>
     <row r="68" ht="15.75" customHeight="1" s="12"/>
     <row r="69" ht="15.75" customHeight="1" s="12"/>
     <row r="70" ht="15.75" customHeight="1" s="12"/>

</xml_diff>

<commit_message>
Auto-cleanup: Remove temp files committed by mistake
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX18"/>
+  <dimension ref="A1:AX24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="9" min="1" max="2"/>
@@ -1617,7 +1617,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Liu et al.</t>
+          <t>LIU Songbo &amp; LI Yuhui</t>
         </is>
       </c>
       <c r="K12" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>High-tech park employees</t>
+          <t>employees from high-tech enterprises</t>
         </is>
       </c>
       <c r="AA12" t="n">
@@ -1662,10 +1662,14 @@
       </c>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
-        </is>
-      </c>
-      <c r="AG12" t="inlineStr"/>
+          <t>采用的是 Marrone 等(2007)开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>5 items adapted from Marrone et al. (2007) 6-item scale, 1 item deleted</t>
+        </is>
+      </c>
       <c r="AH12" t="n">
         <v>999</v>
       </c>
@@ -1675,8 +1679,10 @@
       <c r="AJ12" t="n">
         <v>999</v>
       </c>
-      <c r="AK12" t="n">
-        <v>999</v>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
       </c>
       <c r="AM12" t="inlineStr">
         <is>
@@ -1690,7 +1696,7 @@
       </c>
       <c r="AO12" t="inlineStr">
         <is>
-          <t>员工跨界行为</t>
+          <t>Employee boundary-spanning behavior</t>
         </is>
       </c>
       <c r="AP12" t="n">
@@ -1704,7 +1710,7 @@
       </c>
       <c r="AS12" t="inlineStr">
         <is>
-          <t>员工年龄</t>
+          <t>Employee Age</t>
         </is>
       </c>
       <c r="AT12" t="n">
@@ -1758,7 +1764,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Liu et al.</t>
+          <t>LIU Songbo &amp; LI Yuhui</t>
         </is>
       </c>
       <c r="K13" t="n">
@@ -1784,7 +1790,7 @@
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>High-tech park employees</t>
+          <t>employees from high-tech enterprises</t>
         </is>
       </c>
       <c r="AA13" t="n">
@@ -1803,10 +1809,14 @@
       </c>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
-        </is>
-      </c>
-      <c r="AG13" t="inlineStr"/>
+          <t>采用的是 Marrone 等(2007)开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>5 items adapted from Marrone et al. (2007) 6-item scale, 1 item deleted</t>
+        </is>
+      </c>
       <c r="AH13" t="n">
         <v>999</v>
       </c>
@@ -1816,8 +1826,10 @@
       <c r="AJ13" t="n">
         <v>999</v>
       </c>
-      <c r="AK13" t="n">
-        <v>999</v>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
       </c>
       <c r="AM13" t="inlineStr">
         <is>
@@ -1826,12 +1838,12 @@
       </c>
       <c r="AN13" t="inlineStr">
         <is>
-          <t>1 = male, 0 = female</t>
+          <t>0 = Female, 1 = Male</t>
         </is>
       </c>
       <c r="AO13" t="inlineStr">
         <is>
-          <t>员工跨界行为</t>
+          <t>Employee boundary-spanning behavior</t>
         </is>
       </c>
       <c r="AP13" t="n">
@@ -1845,7 +1857,7 @@
       </c>
       <c r="AS13" t="inlineStr">
         <is>
-          <t>员工性别</t>
+          <t>Employee Gender</t>
         </is>
       </c>
       <c r="AT13" t="n">
@@ -1899,7 +1911,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Liu et al.</t>
+          <t>LIU Songbo &amp; LI Yuhui</t>
         </is>
       </c>
       <c r="K14" t="n">
@@ -1925,7 +1937,7 @@
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>High-tech park employees</t>
+          <t>employees from high-tech enterprises</t>
         </is>
       </c>
       <c r="AA14" t="n">
@@ -1944,10 +1956,14 @@
       </c>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
-        </is>
-      </c>
-      <c r="AG14" t="inlineStr"/>
+          <t>采用的是 Marrone 等(2007)开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>5 items adapted from Marrone et al. (2007) 6-item scale, 1 item deleted</t>
+        </is>
+      </c>
       <c r="AH14" t="n">
         <v>999</v>
       </c>
@@ -1957,8 +1973,10 @@
       <c r="AJ14" t="n">
         <v>999</v>
       </c>
-      <c r="AK14" t="n">
-        <v>999</v>
+      <c r="AK14" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
       </c>
       <c r="AM14" t="inlineStr">
         <is>
@@ -1967,12 +1985,12 @@
       </c>
       <c r="AN14" t="inlineStr">
         <is>
-          <t>1 (high school and below) to 6 (doctoral degree)</t>
+          <t>Coded 1 (High school and below) to 6 (Doctorate)</t>
         </is>
       </c>
       <c r="AO14" t="inlineStr">
         <is>
-          <t>员工跨界行为</t>
+          <t>Employee boundary-spanning behavior</t>
         </is>
       </c>
       <c r="AP14" t="n">
@@ -1986,7 +2004,7 @@
       </c>
       <c r="AS14" t="inlineStr">
         <is>
-          <t>教育程度</t>
+          <t>Employee Education</t>
         </is>
       </c>
       <c r="AT14" t="n">
@@ -2040,7 +2058,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Liu et al.</t>
+          <t>LIU Songbo &amp; LI Yuhui</t>
         </is>
       </c>
       <c r="K15" t="n">
@@ -2066,7 +2084,7 @@
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>High-tech park employees</t>
+          <t>employees from high-tech enterprises</t>
         </is>
       </c>
       <c r="AA15" t="n">
@@ -2085,10 +2103,14 @@
       </c>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
-        </is>
-      </c>
-      <c r="AG15" t="inlineStr"/>
+          <t>采用的是 Marrone 等(2007)开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>5 items adapted from Marrone et al. (2007) 6-item scale, 1 item deleted</t>
+        </is>
+      </c>
       <c r="AH15" t="n">
         <v>999</v>
       </c>
@@ -2098,8 +2120,10 @@
       <c r="AJ15" t="n">
         <v>999</v>
       </c>
-      <c r="AK15" t="n">
-        <v>999</v>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
       </c>
       <c r="AM15" t="inlineStr">
         <is>
@@ -2113,7 +2137,7 @@
       </c>
       <c r="AO15" t="inlineStr">
         <is>
-          <t>员工跨界行为</t>
+          <t>Employee boundary-spanning behavior</t>
         </is>
       </c>
       <c r="AP15" t="n">
@@ -2127,7 +2151,7 @@
       </c>
       <c r="AS15" t="inlineStr">
         <is>
-          <t>本团队工作时间</t>
+          <t>Team Tenure</t>
         </is>
       </c>
       <c r="AT15" t="n">
@@ -2181,7 +2205,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Liu et al.</t>
+          <t>LIU Songbo &amp; LI Yuhui</t>
         </is>
       </c>
       <c r="K16" t="n">
@@ -2207,7 +2231,7 @@
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>High-tech park employees</t>
+          <t>employees from high-tech enterprises</t>
         </is>
       </c>
       <c r="AA16" t="n">
@@ -2226,10 +2250,14 @@
       </c>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
-        </is>
-      </c>
-      <c r="AG16" t="inlineStr"/>
+          <t>采用的是 Marrone 等(2007)开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>5 items adapted from Marrone et al. (2007) 6-item scale, 1 item deleted</t>
+        </is>
+      </c>
       <c r="AH16" t="n">
         <v>3</v>
       </c>
@@ -2246,13 +2274,13 @@
       </c>
       <c r="AM16" t="inlineStr">
         <is>
-          <t>集体主义 采用 Ilies, Wagner 和Morgeson (2007) 使用过的量表 , 共3个条目 , 比如 “比起独自工作来说 , 我更愿意和同事一起工作 ”等。</t>
+          <t>集体主义   采用 Ilies, Wagner 和Morgeson (2007) 使用过的量表 , 共3个条目 , 比如 “比起独自工作来说 , 我更愿意和同事一起工作 ”等。在本研究中使用 Likert 7 点测量方法 , 1表示 “非常不同意 ”, 7表示 “非常同意 ”。</t>
         </is>
       </c>
       <c r="AN16" t="inlineStr"/>
       <c r="AO16" t="inlineStr">
         <is>
-          <t>员工跨界行为</t>
+          <t>Employee boundary-spanning behavior</t>
         </is>
       </c>
       <c r="AP16" t="n">
@@ -2266,7 +2294,7 @@
       </c>
       <c r="AS16" t="inlineStr">
         <is>
-          <t>集体主义导向</t>
+          <t>Collectivism orientation</t>
         </is>
       </c>
       <c r="AT16" t="n">
@@ -2320,7 +2348,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Liu et al.</t>
+          <t>LIU Songbo &amp; LI Yuhui</t>
         </is>
       </c>
       <c r="K17" t="n">
@@ -2346,7 +2374,7 @@
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>High-tech park employees</t>
+          <t>employees from high-tech enterprises</t>
         </is>
       </c>
       <c r="AA17" t="n">
@@ -2365,10 +2393,14 @@
       </c>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
-        </is>
-      </c>
-      <c r="AG17" t="inlineStr"/>
+          <t>采用的是 Marrone 等(2007)开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>5 items adapted from Marrone et al. (2007) 6-item scale, 1 item deleted</t>
+        </is>
+      </c>
       <c r="AH17" t="n">
         <v>2</v>
       </c>
@@ -2385,17 +2417,13 @@
       </c>
       <c r="AM17" t="inlineStr">
         <is>
-          <t>咨询网络中心性 采用的是 Sparrowe 等(2001) 采用的点入中心性 (in-degree centrality, Borgatti, Everett, &amp; Freeman, 1992) 的测量方法。为了收集整体网络数据 , 我们在每个团队中都列上了所有成员的名字 , 然后要求员工对其同事进行评价。量表共 2个条目 , 比如 “你向 (某某 )寻求有关工作的帮助或建议吗 ”。我们关心的是这种关系的强度 (strength), 所以通过 Likert 5 点来进行测量 , 1表示 “从不 ”, 5表示 “总是 ”。</t>
-        </is>
-      </c>
-      <c r="AN17" t="inlineStr">
-        <is>
-          <t>Advice network centrality</t>
-        </is>
-      </c>
+          <t>咨询网络中心性   采用的是 Sparrowe 等(2001) 采用的点入中心性 (in-degree centrality, Borgatti, Everett, &amp; Freeman, 1992) 的测量方法。为了收集整体 network 数据 , 我们在每个团队中都列上了所有成员的名字 , 然后要求员工对其同事进行评价。量表共 2个条目 , 比如 “你向 (某某 )寻求有关工作的帮助或建议吗 ”。我们关心的是这种关系的强度 (strength), 所以通过 Likert 5 点来进行测量 , 1表示 “从不 ”, 5表示“总是 ”。所谓点入中心性是相对于点出中心性 (out-degree centrality, 员工本人评价的与自己其他成员的关系 )而言的 , 指的是每个员工来自团队中其他成员评价的网络地位的均值。</t>
+        </is>
+      </c>
+      <c r="AN17" t="inlineStr"/>
       <c r="AO17" t="inlineStr">
         <is>
-          <t>员工跨界行为</t>
+          <t>Employee boundary-spanning behavior</t>
         </is>
       </c>
       <c r="AP17" t="n">
@@ -2409,7 +2437,7 @@
       </c>
       <c r="AS17" t="inlineStr">
         <is>
-          <t>网络中心性</t>
+          <t>Advice network centrality</t>
         </is>
       </c>
       <c r="AT17" t="n">
@@ -2463,7 +2491,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Liu et al.</t>
+          <t>LIU Songbo &amp; LI Yuhui</t>
         </is>
       </c>
       <c r="K18" t="n">
@@ -2489,7 +2517,7 @@
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>High-tech park employees</t>
+          <t>employees from high-tech enterprises</t>
         </is>
       </c>
       <c r="AA18" t="n">
@@ -2508,10 +2536,14 @@
       </c>
       <c r="AF18" t="inlineStr">
         <is>
-          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
-        </is>
-      </c>
-      <c r="AG18" t="inlineStr"/>
+          <t>采用的是 Marrone 等(2007)开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>5 items adapted from Marrone et al. (2007) 6-item scale, 1 item deleted</t>
+        </is>
+      </c>
       <c r="AH18" t="n">
         <v>4</v>
       </c>
@@ -2528,13 +2560,13 @@
       </c>
       <c r="AM18" t="inlineStr">
         <is>
-          <t>任务绩效 采用的是 Liden, Wayne 和Stilwell (1993) 开发的量表 , 共4个条目 , 比如 “这名员工能够充分完成分配的任务 ”等, 由领导填写。</t>
+          <t>任务绩效  采用的是 Liden, Wayne 和Stilwell (1993) 开发的量表 , 共4个条目 , 比如 “这名员工能够充分完成分配的任务 ”等, 由领导填写。在本研究中使用 Likert7 点测量方法 , 1表示 “非常不同意 ”, 7表示 “非常同意 ”。</t>
         </is>
       </c>
       <c r="AN18" t="inlineStr"/>
       <c r="AO18" t="inlineStr">
         <is>
-          <t>员工跨界行为</t>
+          <t>Employee boundary-spanning behavior</t>
         </is>
       </c>
       <c r="AP18" t="n">
@@ -2548,7 +2580,7 @@
       </c>
       <c r="AS18" t="inlineStr">
         <is>
-          <t>任务绩效</t>
+          <t>Task performance</t>
         </is>
       </c>
       <c r="AT18" t="n">
@@ -2564,12 +2596,842 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1" s="9"/>
-    <row r="20" ht="15.75" customHeight="1" s="9"/>
-    <row r="21" ht="15.75" customHeight="1" s="9"/>
-    <row r="22" ht="15.75" customHeight="1" s="9"/>
-    <row r="23" ht="15.75" customHeight="1" s="9"/>
-    <row r="24" ht="15.75" customHeight="1" s="9"/>
+    <row r="19" ht="15.75" customHeight="1" s="9">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>BSMA0004</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BSMA0004.1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>BSMA0004.1.2</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Acta Psychologica Sinica</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Liu et al.</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>2014</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>2 = Longitudinal/time-lagged</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V19" t="n">
+        <v>292</v>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>High-tech park employees</t>
+        </is>
+      </c>
+      <c r="AA19" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AH19" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>999</v>
+      </c>
+      <c r="AM19" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+      <c r="AN19" t="inlineStr">
+        <is>
+          <t>1 = male, 0 = female</t>
+        </is>
+      </c>
+      <c r="AO19" t="inlineStr">
+        <is>
+          <t>员工跨界行为</t>
+        </is>
+      </c>
+      <c r="AP19" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="AQ19" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AR19" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t>员工性别</t>
+        </is>
+      </c>
+      <c r="AT19" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="AU19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV19" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW19" t="n">
+        <v>-0.06</v>
+      </c>
+    </row>
+    <row r="20" ht="15.75" customHeight="1" s="9">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>BSMA0004</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BSMA0004.1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>BSMA0004.1.3</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Acta Psychologica Sinica</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Liu et al.</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>2014</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>2 = Longitudinal/time-lagged</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V20" t="n">
+        <v>292</v>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>High-tech park employees</t>
+        </is>
+      </c>
+      <c r="AA20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AH20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AM20" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>1 (high school and below) to 6 (doctoral degree)</t>
+        </is>
+      </c>
+      <c r="AO20" t="inlineStr">
+        <is>
+          <t>员工跨界行为</t>
+        </is>
+      </c>
+      <c r="AP20" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="AQ20" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AR20" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="AS20" t="inlineStr">
+        <is>
+          <t>教育程度</t>
+        </is>
+      </c>
+      <c r="AT20" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="AU20" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="AV20" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW20" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1" s="9">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>BSMA0004</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>BSMA0004.1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>BSMA0004.1.4</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Acta Psychologica Sinica</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Liu et al.</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>2014</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>2 = Longitudinal/time-lagged</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V21" t="n">
+        <v>292</v>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>High-tech park employees</t>
+        </is>
+      </c>
+      <c r="AA21" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AH21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AM21" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>Months</t>
+        </is>
+      </c>
+      <c r="AO21" t="inlineStr">
+        <is>
+          <t>员工跨界行为</t>
+        </is>
+      </c>
+      <c r="AP21" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="AQ21" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AR21" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="AS21" t="inlineStr">
+        <is>
+          <t>本团队工作时间</t>
+        </is>
+      </c>
+      <c r="AT21" t="n">
+        <v>20.64</v>
+      </c>
+      <c r="AU21" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="AV21" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW21" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1" s="9">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>BSMA0004</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>BSMA0004.1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>BSMA0004.1.5</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Acta Psychologica Sinica</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Liu et al.</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>2014</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>2 = Longitudinal/time-lagged</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V22" t="n">
+        <v>292</v>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>High-tech park employees</t>
+        </is>
+      </c>
+      <c r="AA22" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AH22" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ22" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK22" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AM22" t="inlineStr">
+        <is>
+          <t>集体主义 采用 Ilies, Wagner 和Morgeson (2007) 使用过的量表 , 共3个条目 , 比如 “比起独自工作来说 , 我更愿意和同事一起工作 ”等。</t>
+        </is>
+      </c>
+      <c r="AO22" t="inlineStr">
+        <is>
+          <t>员工跨界行为</t>
+        </is>
+      </c>
+      <c r="AP22" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AR22" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="AS22" t="inlineStr">
+        <is>
+          <t>集体主义导向</t>
+        </is>
+      </c>
+      <c r="AT22" t="n">
+        <v>5.84</v>
+      </c>
+      <c r="AU22" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="AV22" t="n">
+        <v>0.891</v>
+      </c>
+      <c r="AW22" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="9">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>BSMA0004</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>BSMA0004.1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>BSMA0004.1.6</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Acta Psychologica Sinica</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Liu et al.</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>2014</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>2 = Longitudinal/time-lagged</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V23" t="n">
+        <v>292</v>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>High-tech park employees</t>
+        </is>
+      </c>
+      <c r="AA23" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AH23" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ23" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK23" t="inlineStr">
+        <is>
+          <t>3 = Others</t>
+        </is>
+      </c>
+      <c r="AM23" t="inlineStr">
+        <is>
+          <t>咨询网络中心性 采用的是 Sparrowe 等(2001) 采用的点入中心性 (in-degree centrality, Borgatti, Everett, &amp; Freeman, 1992) 的测量方法。为了收集整体网络数据 , 我们在每个团队中都列上了所有成员的名字 , 然后要求员工对其同事进行评价。量表共 2个条目 , 比如 “你向 (某某 )寻求有关工作的帮助或建议吗 ”。我们关心的是这种关系的强度 (strength), 所以通过 Likert 5 点来进行测量 , 1表示 “从不 ”, 5表示 “总是 ”。</t>
+        </is>
+      </c>
+      <c r="AN23" t="inlineStr">
+        <is>
+          <t>Advice network centrality</t>
+        </is>
+      </c>
+      <c r="AO23" t="inlineStr">
+        <is>
+          <t>员工跨界行为</t>
+        </is>
+      </c>
+      <c r="AP23" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="AQ23" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AR23" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="AS23" t="inlineStr">
+        <is>
+          <t>网络中心性</t>
+        </is>
+      </c>
+      <c r="AT23" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="AU23" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="AV23" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="AW23" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="9">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>BSMA0004</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>BSMA0004.1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>BSMA0004.1.7</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Acta Psychologica Sinica</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Liu et al.</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
+        <v>2014</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>1 = Journal article</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>2 = Longitudinal/time-lagged</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>1 = No (domestic only)</t>
+        </is>
+      </c>
+      <c r="V24" t="n">
+        <v>292</v>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>High-tech park employees</t>
+        </is>
+      </c>
+      <c r="AA24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>1 = Self</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
+        </is>
+      </c>
+      <c r="AH24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AI24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ24" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK24" t="inlineStr">
+        <is>
+          <t>2 = Supervisor</t>
+        </is>
+      </c>
+      <c r="AM24" t="inlineStr">
+        <is>
+          <t>任务绩效 采用的是 Liden, Wayne 和Stilwell (1993) 开发的量表 , 共4个条目 , 比如 “这名员工能够充分完成分配的任务 ”等, 由领导填写。</t>
+        </is>
+      </c>
+      <c r="AO24" t="inlineStr">
+        <is>
+          <t>员工跨界行为</t>
+        </is>
+      </c>
+      <c r="AP24" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AR24" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="AS24" t="inlineStr">
+        <is>
+          <t>任务绩效</t>
+        </is>
+      </c>
+      <c r="AT24" t="n">
+        <v>5.57</v>
+      </c>
+      <c r="AU24" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="AV24" t="n">
+        <v>0.919</v>
+      </c>
+      <c r="AW24" t="n">
+        <v>0.31</v>
+      </c>
+    </row>
     <row r="25" ht="15.75" customHeight="1" s="9"/>
     <row r="26" ht="15.75" customHeight="1" s="9"/>
     <row r="27" ht="15.75" customHeight="1" s="9"/>

</xml_diff>

<commit_message>
Clean up duplicate Chinese rows for BSMA0004
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX24"/>
+  <dimension ref="A1:AX18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.25" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.5625" customWidth="1" style="9" min="1" max="2"/>
@@ -2277,7 +2277,6 @@
           <t>集体主义   采用 Ilies, Wagner 和Morgeson (2007) 使用过的量表 , 共3个条目 , 比如 “比起独自工作来说 , 我更愿意和同事一起工作 ”等。在本研究中使用 Likert 7 点测量方法 , 1表示 “非常不同意 ”, 7表示 “非常同意 ”。</t>
         </is>
       </c>
-      <c r="AN16" t="inlineStr"/>
       <c r="AO16" t="inlineStr">
         <is>
           <t>Employee boundary-spanning behavior</t>
@@ -2420,7 +2419,6 @@
           <t>咨询网络中心性   采用的是 Sparrowe 等(2001) 采用的点入中心性 (in-degree centrality, Borgatti, Everett, &amp; Freeman, 1992) 的测量方法。为了收集整体 network 数据 , 我们在每个团队中都列上了所有成员的名字 , 然后要求员工对其同事进行评价。量表共 2个条目 , 比如 “你向 (某某 )寻求有关工作的帮助或建议吗 ”。我们关心的是这种关系的强度 (strength), 所以通过 Likert 5 点来进行测量 , 1表示 “从不 ”, 5表示“总是 ”。所谓点入中心性是相对于点出中心性 (out-degree centrality, 员工本人评价的与自己其他成员的关系 )而言的 , 指的是每个员工来自团队中其他成员评价的网络地位的均值。</t>
         </is>
       </c>
-      <c r="AN17" t="inlineStr"/>
       <c r="AO17" t="inlineStr">
         <is>
           <t>Employee boundary-spanning behavior</t>
@@ -2563,7 +2561,6 @@
           <t>任务绩效  采用的是 Liden, Wayne 和Stilwell (1993) 开发的量表 , 共4个条目 , 比如 “这名员工能够充分完成分配的任务 ”等, 由领导填写。在本研究中使用 Likert7 点测量方法 , 1表示 “非常不同意 ”, 7表示 “非常同意 ”。</t>
         </is>
       </c>
-      <c r="AN18" t="inlineStr"/>
       <c r="AO18" t="inlineStr">
         <is>
           <t>Employee boundary-spanning behavior</t>
@@ -2596,842 +2593,12 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1" s="9">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>BSMA0004</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>BSMA0004.1</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>BSMA0004.1.2</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>Acta Psychologica Sinica</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Liu et al.</t>
-        </is>
-      </c>
-      <c r="K19" t="n">
-        <v>2014</v>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>2 = Longitudinal/time-lagged</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V19" t="n">
-        <v>292</v>
-      </c>
-      <c r="Z19" t="inlineStr">
-        <is>
-          <t>High-tech park employees</t>
-        </is>
-      </c>
-      <c r="AA19" t="n">
-        <v>5</v>
-      </c>
-      <c r="AB19" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC19" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD19" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AF19" t="inlineStr">
-        <is>
-          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
-        </is>
-      </c>
-      <c r="AH19" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI19" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ19" t="n">
-        <v>999</v>
-      </c>
-      <c r="AK19" t="n">
-        <v>999</v>
-      </c>
-      <c r="AM19" t="inlineStr">
-        <is>
-          <t>999</t>
-        </is>
-      </c>
-      <c r="AN19" t="inlineStr">
-        <is>
-          <t>1 = male, 0 = female</t>
-        </is>
-      </c>
-      <c r="AO19" t="inlineStr">
-        <is>
-          <t>员工跨界行为</t>
-        </is>
-      </c>
-      <c r="AP19" t="n">
-        <v>4.98</v>
-      </c>
-      <c r="AQ19" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="AR19" t="n">
-        <v>0.869</v>
-      </c>
-      <c r="AS19" t="inlineStr">
-        <is>
-          <t>员工性别</t>
-        </is>
-      </c>
-      <c r="AT19" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="AU19" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AV19" t="n">
-        <v>999</v>
-      </c>
-      <c r="AW19" t="n">
-        <v>-0.06</v>
-      </c>
-    </row>
-    <row r="20" ht="15.75" customHeight="1" s="9">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>BSMA0004</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>BSMA0004.1</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>BSMA0004.1.3</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>Acta Psychologica Sinica</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Liu et al.</t>
-        </is>
-      </c>
-      <c r="K20" t="n">
-        <v>2014</v>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>2 = Longitudinal/time-lagged</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V20" t="n">
-        <v>292</v>
-      </c>
-      <c r="Z20" t="inlineStr">
-        <is>
-          <t>High-tech park employees</t>
-        </is>
-      </c>
-      <c r="AA20" t="n">
-        <v>5</v>
-      </c>
-      <c r="AB20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC20" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD20" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AF20" t="inlineStr">
-        <is>
-          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
-        </is>
-      </c>
-      <c r="AH20" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI20" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ20" t="n">
-        <v>999</v>
-      </c>
-      <c r="AK20" t="n">
-        <v>999</v>
-      </c>
-      <c r="AM20" t="inlineStr">
-        <is>
-          <t>999</t>
-        </is>
-      </c>
-      <c r="AN20" t="inlineStr">
-        <is>
-          <t>1 (high school and below) to 6 (doctoral degree)</t>
-        </is>
-      </c>
-      <c r="AO20" t="inlineStr">
-        <is>
-          <t>员工跨界行为</t>
-        </is>
-      </c>
-      <c r="AP20" t="n">
-        <v>4.98</v>
-      </c>
-      <c r="AQ20" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="AR20" t="n">
-        <v>0.869</v>
-      </c>
-      <c r="AS20" t="inlineStr">
-        <is>
-          <t>教育程度</t>
-        </is>
-      </c>
-      <c r="AT20" t="n">
-        <v>3.28</v>
-      </c>
-      <c r="AU20" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="AV20" t="n">
-        <v>999</v>
-      </c>
-      <c r="AW20" t="n">
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1" s="9">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>BSMA0004</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>BSMA0004.1</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>BSMA0004.1.4</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Acta Psychologica Sinica</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Liu et al.</t>
-        </is>
-      </c>
-      <c r="K21" t="n">
-        <v>2014</v>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>2 = Longitudinal/time-lagged</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V21" t="n">
-        <v>292</v>
-      </c>
-      <c r="Z21" t="inlineStr">
-        <is>
-          <t>High-tech park employees</t>
-        </is>
-      </c>
-      <c r="AA21" t="n">
-        <v>5</v>
-      </c>
-      <c r="AB21" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC21" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD21" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AF21" t="inlineStr">
-        <is>
-          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
-        </is>
-      </c>
-      <c r="AH21" t="n">
-        <v>999</v>
-      </c>
-      <c r="AI21" t="n">
-        <v>999</v>
-      </c>
-      <c r="AJ21" t="n">
-        <v>999</v>
-      </c>
-      <c r="AK21" t="n">
-        <v>999</v>
-      </c>
-      <c r="AM21" t="inlineStr">
-        <is>
-          <t>999</t>
-        </is>
-      </c>
-      <c r="AN21" t="inlineStr">
-        <is>
-          <t>Months</t>
-        </is>
-      </c>
-      <c r="AO21" t="inlineStr">
-        <is>
-          <t>员工跨界行为</t>
-        </is>
-      </c>
-      <c r="AP21" t="n">
-        <v>4.98</v>
-      </c>
-      <c r="AQ21" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="AR21" t="n">
-        <v>0.869</v>
-      </c>
-      <c r="AS21" t="inlineStr">
-        <is>
-          <t>本团队工作时间</t>
-        </is>
-      </c>
-      <c r="AT21" t="n">
-        <v>20.64</v>
-      </c>
-      <c r="AU21" t="n">
-        <v>18.47</v>
-      </c>
-      <c r="AV21" t="n">
-        <v>999</v>
-      </c>
-      <c r="AW21" t="n">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1" s="9">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>BSMA0004</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>BSMA0004.1</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>BSMA0004.1.5</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Acta Psychologica Sinica</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Liu et al.</t>
-        </is>
-      </c>
-      <c r="K22" t="n">
-        <v>2014</v>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>2 = Longitudinal/time-lagged</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V22" t="n">
-        <v>292</v>
-      </c>
-      <c r="Z22" t="inlineStr">
-        <is>
-          <t>High-tech park employees</t>
-        </is>
-      </c>
-      <c r="AA22" t="n">
-        <v>5</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC22" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD22" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AF22" t="inlineStr">
-        <is>
-          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
-        </is>
-      </c>
-      <c r="AH22" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI22" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ22" t="n">
-        <v>7</v>
-      </c>
-      <c r="AK22" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AM22" t="inlineStr">
-        <is>
-          <t>集体主义 采用 Ilies, Wagner 和Morgeson (2007) 使用过的量表 , 共3个条目 , 比如 “比起独自工作来说 , 我更愿意和同事一起工作 ”等。</t>
-        </is>
-      </c>
-      <c r="AO22" t="inlineStr">
-        <is>
-          <t>员工跨界行为</t>
-        </is>
-      </c>
-      <c r="AP22" t="n">
-        <v>4.98</v>
-      </c>
-      <c r="AQ22" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="AR22" t="n">
-        <v>0.869</v>
-      </c>
-      <c r="AS22" t="inlineStr">
-        <is>
-          <t>集体主义导向</t>
-        </is>
-      </c>
-      <c r="AT22" t="n">
-        <v>5.84</v>
-      </c>
-      <c r="AU22" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="AV22" t="n">
-        <v>0.891</v>
-      </c>
-      <c r="AW22" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1" s="9">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>BSMA0004</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>BSMA0004.1</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>BSMA0004.1.6</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>Acta Psychologica Sinica</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Liu et al.</t>
-        </is>
-      </c>
-      <c r="K23" t="n">
-        <v>2014</v>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>2 = Longitudinal/time-lagged</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V23" t="n">
-        <v>292</v>
-      </c>
-      <c r="Z23" t="inlineStr">
-        <is>
-          <t>High-tech park employees</t>
-        </is>
-      </c>
-      <c r="AA23" t="n">
-        <v>5</v>
-      </c>
-      <c r="AB23" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC23" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD23" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AF23" t="inlineStr">
-        <is>
-          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
-        </is>
-      </c>
-      <c r="AH23" t="n">
-        <v>2</v>
-      </c>
-      <c r="AI23" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ23" t="n">
-        <v>5</v>
-      </c>
-      <c r="AK23" t="inlineStr">
-        <is>
-          <t>3 = Others</t>
-        </is>
-      </c>
-      <c r="AM23" t="inlineStr">
-        <is>
-          <t>咨询网络中心性 采用的是 Sparrowe 等(2001) 采用的点入中心性 (in-degree centrality, Borgatti, Everett, &amp; Freeman, 1992) 的测量方法。为了收集整体网络数据 , 我们在每个团队中都列上了所有成员的名字 , 然后要求员工对其同事进行评价。量表共 2个条目 , 比如 “你向 (某某 )寻求有关工作的帮助或建议吗 ”。我们关心的是这种关系的强度 (strength), 所以通过 Likert 5 点来进行测量 , 1表示 “从不 ”, 5表示 “总是 ”。</t>
-        </is>
-      </c>
-      <c r="AN23" t="inlineStr">
-        <is>
-          <t>Advice network centrality</t>
-        </is>
-      </c>
-      <c r="AO23" t="inlineStr">
-        <is>
-          <t>员工跨界行为</t>
-        </is>
-      </c>
-      <c r="AP23" t="n">
-        <v>4.98</v>
-      </c>
-      <c r="AQ23" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="AR23" t="n">
-        <v>0.869</v>
-      </c>
-      <c r="AS23" t="inlineStr">
-        <is>
-          <t>网络中心性</t>
-        </is>
-      </c>
-      <c r="AT23" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="AU23" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="AV23" t="n">
-        <v>0.869</v>
-      </c>
-      <c r="AW23" t="n">
-        <v>0.27</v>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" s="9">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>BSMA0004</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>BSMA0004.1</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>BSMA0004.1.7</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>A Longitudinal Study on the Impact Mechanism of Employees’ Boundary Spanning Behavior: Roles of Centrality and Collectivism</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>Acta Psychologica Sinica</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Liu et al.</t>
-        </is>
-      </c>
-      <c r="K24" t="n">
-        <v>2014</v>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>1 = Journal article</t>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>2 = Longitudinal/time-lagged</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>1 = No (domestic only)</t>
-        </is>
-      </c>
-      <c r="V24" t="n">
-        <v>292</v>
-      </c>
-      <c r="Z24" t="inlineStr">
-        <is>
-          <t>High-tech park employees</t>
-        </is>
-      </c>
-      <c r="AA24" t="n">
-        <v>5</v>
-      </c>
-      <c r="AB24" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC24" t="n">
-        <v>7</v>
-      </c>
-      <c r="AD24" t="inlineStr">
-        <is>
-          <t>1 = Self</t>
-        </is>
-      </c>
-      <c r="AF24" t="inlineStr">
-        <is>
-          <t>员工的跨界行为 采用的是 Marrone 等(2007) 开发的量表。原量表共 6个条目 , 我们删除了原量表中专门针对样本 (咨询团队 )特点设计的 1个条目 , 所以共 5个条目 , 比如 “我会从团队外部人那里为我们团队寻求建议 ”等。</t>
-        </is>
-      </c>
-      <c r="AH24" t="n">
-        <v>4</v>
-      </c>
-      <c r="AI24" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ24" t="n">
-        <v>7</v>
-      </c>
-      <c r="AK24" t="inlineStr">
-        <is>
-          <t>2 = Supervisor</t>
-        </is>
-      </c>
-      <c r="AM24" t="inlineStr">
-        <is>
-          <t>任务绩效 采用的是 Liden, Wayne 和Stilwell (1993) 开发的量表 , 共4个条目 , 比如 “这名员工能够充分完成分配的任务 ”等, 由领导填写。</t>
-        </is>
-      </c>
-      <c r="AO24" t="inlineStr">
-        <is>
-          <t>员工跨界行为</t>
-        </is>
-      </c>
-      <c r="AP24" t="n">
-        <v>4.98</v>
-      </c>
-      <c r="AQ24" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="AR24" t="n">
-        <v>0.869</v>
-      </c>
-      <c r="AS24" t="inlineStr">
-        <is>
-          <t>任务绩效</t>
-        </is>
-      </c>
-      <c r="AT24" t="n">
-        <v>5.57</v>
-      </c>
-      <c r="AU24" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="AV24" t="n">
-        <v>0.919</v>
-      </c>
-      <c r="AW24" t="n">
-        <v>0.31</v>
-      </c>
-    </row>
+    <row r="19" ht="15.75" customHeight="1" s="9"/>
+    <row r="20" ht="15.75" customHeight="1" s="9"/>
+    <row r="21" ht="15.75" customHeight="1" s="9"/>
+    <row r="22" ht="15.75" customHeight="1" s="9"/>
+    <row r="23" ht="15.75" customHeight="1" s="9"/>
+    <row r="24" ht="15.75" customHeight="1" s="9"/>
     <row r="25" ht="15.75" customHeight="1" s="9"/>
     <row r="26" ht="15.75" customHeight="1" s="9"/>
     <row r="27" ht="15.75" customHeight="1" s="9"/>

</xml_diff>

<commit_message>
Learn: Exclusion code 99 with Notes, universal Excel insertion rule
</commit_message>
<xml_diff>
--- a/BSMA_Master_Coding_Sheet.xlsx
+++ b/BSMA_Master_Coding_Sheet.xlsx
@@ -982,7 +982,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Firm-level boundary spanning (Precedent #002): Focal spanner is the firm, not an individual.</t>
+          <t>99 = Other (specify in Notes)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1002,6 +1002,11 @@
       </c>
       <c r="K6" t="n">
         <v>2025</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Firm-level boundary spanning (not individual-level). Focal spanner is the firm.</t>
+        </is>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1" s="9"/>
@@ -1023,7 +1028,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Team-level boundary spanning: Focal spanner is the team (N=49 interorganizational teams), not an individual.</t>
+          <t>99 = Other (specify in Notes)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1043,6 +1048,11 @@
       </c>
       <c r="K8" t="n">
         <v>2011</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Team-level boundary spanning (not individual-level). Focal spanner is the team (N=49).</t>
+        </is>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1" s="9"/>

</xml_diff>